<commit_message>
weekly gannt chart update
</commit_message>
<xml_diff>
--- a/Documentation/GanntChart/BattleNationsGanntChart.xlsx
+++ b/Documentation/GanntChart/BattleNationsGanntChart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jreig\git\BattleNations\Documentation\GanntChart\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{34C683D4-32F6-4647-8681-0B1E686158EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{142F7CFD-1580-4713-AC11-3E3E6C5B1251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="212">
   <si>
     <t/>
   </si>
@@ -287,9 +287,6 @@
     <t>17-Apr-2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Update whatever requests we get from customer </t>
-  </si>
-  <si>
     <t>24-Apr-2026</t>
   </si>
   <si>
@@ -482,9 +479,6 @@
     <t>Completed by</t>
   </si>
   <si>
-    <t>Max</t>
-  </si>
-  <si>
     <t>JD</t>
   </si>
   <si>
@@ -554,12 +548,6 @@
     <t>Look through all files javadocs + polish anywhere needed</t>
   </si>
   <si>
-    <t>Time to complete: 2 hours</t>
-  </si>
-  <si>
-    <t>Prepare for final Presentation</t>
-  </si>
-  <si>
     <t>Display Player owed region percentages on region display (10-Apr-26 - 17-Apr-26)</t>
   </si>
   <si>
@@ -578,9 +566,6 @@
     <t>Prepare for Customer Presentation  (10-Apr-26 - 17-Apr-26)</t>
   </si>
   <si>
-    <t>Prepare for final Presentation (17-Apr-26 - 24-Apr-26)</t>
-  </si>
-  <si>
     <t>MAX</t>
   </si>
   <si>
@@ -620,9 +605,6 @@
     <t>Add Test Section To game Manual</t>
   </si>
   <si>
-    <t>Update whatever requests we get from customer (17-Apr-26 - 22-Apr-26)</t>
-  </si>
-  <si>
     <t>Polish Game + Visuals  (10-Apr-26 - 17-Apr-26)</t>
   </si>
   <si>
@@ -665,20 +647,35 @@
     <t>Add Flow Charts to game Manual</t>
   </si>
   <si>
-    <t xml:space="preserve">Add Images to Game Manual Where Appropriate </t>
-  </si>
-  <si>
     <t>Add Images to Game Manual Where Appropriate (17-Apr-26 - 24-Apr-26)</t>
   </si>
   <si>
     <t>Write Final Test for NeighborService Class (17-Apr-26 - 24-Apr-26)</t>
+  </si>
+  <si>
+    <t>Need max to fix his flow charts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update Customer Requests </t>
+  </si>
+  <si>
+    <t>Update Customer Requests  (17-Apr-26 - 22-Apr-26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add &amp; resize Images to Game Manual Where Appropriate </t>
+  </si>
+  <si>
+    <t>Prepare for Final Presentation</t>
+  </si>
+  <si>
+    <t>Prepare For Final Presentation (22-Apr-26 - 27-Apr-26)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="356" x14ac:knownFonts="1">
+  <fonts count="353" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2803,30 +2800,12 @@
     </font>
     <font>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="149">
+  <fills count="150">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3711,7 +3690,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249977111117893"/>
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -4681,24 +4666,12 @@
     <xf numFmtId="0" fontId="349" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="352" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="353" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="354" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="291" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="146" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="290" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -4711,22 +4684,73 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="355" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="352" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="15" fontId="344" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="344" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="148" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="350" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="146" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="331" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="145" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="311" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="322" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="145" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="219" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="220" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="221" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="222" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="223" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="224" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="225" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="166" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="167" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="168" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="295" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -4827,8 +4851,14 @@
     <xf numFmtId="0" fontId="282" fillId="147" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="283" fillId="147" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="284" fillId="147" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="145" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="160" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="161" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="162" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="172" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -4857,30 +4887,6 @@
     <xf numFmtId="0" fontId="126" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="219" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="220" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="221" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="222" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="223" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="224" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="225" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="145" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4986,41 +4992,20 @@
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="160" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="161" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="162" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="166" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="167" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="168" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="344" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="311" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="146" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="146" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="331" fillId="145" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="148" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="331" fillId="146" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="149" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5368,7 +5353,7 @@
     <col min="2" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="13.1640625" customWidth="1"/>
     <col min="5" max="5" width="17.70703125" customWidth="1"/>
-    <col min="6" max="6" width="10.95703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="11.9140625" style="1" customWidth="1"/>
     <col min="7" max="7" width="3.33203125" customWidth="1"/>
     <col min="9" max="9" width="8.5" customWidth="1"/>
     <col min="10" max="10" width="10.33203125" hidden="1" customWidth="1"/>
@@ -5495,13 +5480,13 @@
       <c r="DF1" s="2"/>
     </row>
     <row r="2" spans="1:110" x14ac:dyDescent="0.8">
-      <c r="A2" s="376" t="s">
+      <c r="A2" s="391" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="377" t="s">
+      <c r="B2" s="392" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="377" t="s">
+      <c r="C2" s="392" t="s">
         <v>0</v>
       </c>
       <c r="D2" s="11"/>
@@ -5510,313 +5495,313 @@
       <c r="G2" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="H2" s="378" t="s">
+      <c r="H2" s="393" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="377" t="s">
+      <c r="I2" s="392" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="377" t="s">
+      <c r="J2" s="392" t="s">
         <v>2</v>
       </c>
-      <c r="K2" s="377" t="s">
+      <c r="K2" s="392" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="377" t="s">
+      <c r="L2" s="392" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="377" t="s">
+      <c r="M2" s="392" t="s">
         <v>2</v>
       </c>
-      <c r="N2" s="377" t="s">
+      <c r="N2" s="392" t="s">
         <v>2</v>
       </c>
-      <c r="O2" s="377" t="s">
+      <c r="O2" s="392" t="s">
         <v>2</v>
       </c>
-      <c r="P2" s="377" t="s">
+      <c r="P2" s="392" t="s">
         <v>2</v>
       </c>
-      <c r="Q2" s="377" t="s">
+      <c r="Q2" s="392" t="s">
         <v>2</v>
       </c>
-      <c r="R2" s="377" t="s">
+      <c r="R2" s="392" t="s">
         <v>2</v>
       </c>
-      <c r="S2" s="377" t="s">
+      <c r="S2" s="392" t="s">
         <v>2</v>
       </c>
-      <c r="T2" s="423" t="s">
+      <c r="T2" s="430" t="s">
         <v>3</v>
       </c>
-      <c r="U2" s="377" t="s">
+      <c r="U2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="V2" s="377" t="s">
+      <c r="V2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="W2" s="377" t="s">
+      <c r="W2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="X2" s="377" t="s">
+      <c r="X2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="Y2" s="377" t="s">
+      <c r="Y2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="Z2" s="377" t="s">
+      <c r="Z2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AA2" s="377" t="s">
+      <c r="AA2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AB2" s="377" t="s">
+      <c r="AB2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AC2" s="377" t="s">
+      <c r="AC2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AD2" s="377" t="s">
+      <c r="AD2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AE2" s="377" t="s">
+      <c r="AE2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AF2" s="377" t="s">
+      <c r="AF2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AG2" s="377" t="s">
+      <c r="AG2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AH2" s="377" t="s">
+      <c r="AH2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AI2" s="377" t="s">
+      <c r="AI2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AJ2" s="377" t="s">
+      <c r="AJ2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AK2" s="377" t="s">
+      <c r="AK2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AL2" s="377" t="s">
+      <c r="AL2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AM2" s="377" t="s">
+      <c r="AM2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AN2" s="377" t="s">
+      <c r="AN2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AO2" s="377" t="s">
+      <c r="AO2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AP2" s="377" t="s">
+      <c r="AP2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AQ2" s="377" t="s">
+      <c r="AQ2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AR2" s="377" t="s">
+      <c r="AR2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AS2" s="377" t="s">
+      <c r="AS2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AT2" s="377" t="s">
+      <c r="AT2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AU2" s="377" t="s">
+      <c r="AU2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AV2" s="377" t="s">
+      <c r="AV2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AW2" s="377" t="s">
+      <c r="AW2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AX2" s="377" t="s">
+      <c r="AX2" s="392" t="s">
         <v>3</v>
       </c>
-      <c r="AY2" s="424" t="s">
+      <c r="AY2" s="431" t="s">
         <v>4</v>
       </c>
-      <c r="AZ2" s="377" t="s">
+      <c r="AZ2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BA2" s="377" t="s">
+      <c r="BA2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BB2" s="377" t="s">
+      <c r="BB2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BC2" s="377" t="s">
+      <c r="BC2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BD2" s="377" t="s">
+      <c r="BD2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BE2" s="377" t="s">
+      <c r="BE2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BF2" s="377" t="s">
+      <c r="BF2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BG2" s="377" t="s">
+      <c r="BG2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BH2" s="377" t="s">
+      <c r="BH2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BI2" s="377" t="s">
+      <c r="BI2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BJ2" s="377" t="s">
+      <c r="BJ2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BK2" s="377" t="s">
+      <c r="BK2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BL2" s="377" t="s">
+      <c r="BL2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BM2" s="377" t="s">
+      <c r="BM2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BN2" s="377" t="s">
+      <c r="BN2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BO2" s="377" t="s">
+      <c r="BO2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BP2" s="377" t="s">
+      <c r="BP2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BQ2" s="377" t="s">
+      <c r="BQ2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BR2" s="377" t="s">
+      <c r="BR2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BS2" s="377" t="s">
+      <c r="BS2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BT2" s="377" t="s">
+      <c r="BT2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BU2" s="377" t="s">
+      <c r="BU2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BV2" s="377" t="s">
+      <c r="BV2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BW2" s="377" t="s">
+      <c r="BW2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BX2" s="377" t="s">
+      <c r="BX2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BY2" s="377" t="s">
+      <c r="BY2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="BZ2" s="377" t="s">
+      <c r="BZ2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="CA2" s="377" t="s">
+      <c r="CA2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="CB2" s="377" t="s">
+      <c r="CB2" s="392" t="s">
         <v>4</v>
       </c>
-      <c r="CC2" s="390" t="s">
+      <c r="CC2" s="397" t="s">
         <v>5</v>
       </c>
-      <c r="CD2" s="377" t="s">
+      <c r="CD2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CE2" s="377" t="s">
+      <c r="CE2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CF2" s="377" t="s">
+      <c r="CF2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CG2" s="377" t="s">
+      <c r="CG2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CH2" s="377" t="s">
+      <c r="CH2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CI2" s="377" t="s">
+      <c r="CI2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CJ2" s="377" t="s">
+      <c r="CJ2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CK2" s="377" t="s">
+      <c r="CK2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CL2" s="377" t="s">
+      <c r="CL2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CM2" s="377" t="s">
+      <c r="CM2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CN2" s="377" t="s">
+      <c r="CN2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CO2" s="377" t="s">
+      <c r="CO2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CP2" s="377" t="s">
+      <c r="CP2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CQ2" s="377" t="s">
+      <c r="CQ2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CR2" s="377" t="s">
+      <c r="CR2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CS2" s="377" t="s">
+      <c r="CS2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CT2" s="377" t="s">
+      <c r="CT2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CU2" s="377" t="s">
+      <c r="CU2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CV2" s="377" t="s">
+      <c r="CV2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CW2" s="377" t="s">
+      <c r="CW2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CX2" s="377" t="s">
+      <c r="CX2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CY2" s="377" t="s">
+      <c r="CY2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="CZ2" s="377" t="s">
+      <c r="CZ2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="DA2" s="377" t="s">
+      <c r="DA2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="DB2" s="377" t="s">
+      <c r="DB2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="DC2" s="377" t="s">
+      <c r="DC2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="DD2" s="377" t="s">
+      <c r="DD2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="DE2" s="377" t="s">
+      <c r="DE2" s="392" t="s">
         <v>5</v>
       </c>
-      <c r="DF2" s="377" t="s">
+      <c r="DF2" s="392" t="s">
         <v>5</v>
       </c>
     </row>
@@ -5831,13 +5816,13 @@
         <v>7</v>
       </c>
       <c r="D3" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="F3" s="17" t="s">
         <v>86</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="F3" s="17" t="s">
-        <v>87</v>
       </c>
       <c r="G3" s="18" t="s">
         <v>0</v>
@@ -6276,7 +6261,7 @@
     </row>
     <row r="5" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A5" s="281" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B5" s="129" t="s">
         <v>40</v>
@@ -6287,23 +6272,23 @@
       <c r="D5" s="131">
         <v>1</v>
       </c>
-      <c r="E5" s="326" t="s">
-        <v>149</v>
+      <c r="E5" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F5" s="132"/>
       <c r="G5" s="133" t="s">
         <v>0</v>
       </c>
-      <c r="H5" s="333" t="s">
-        <v>88</v>
-      </c>
-      <c r="I5" s="379" t="s">
+      <c r="H5" s="336" t="s">
+        <v>87</v>
+      </c>
+      <c r="I5" s="394" t="s">
         <v>42</v>
       </c>
-      <c r="J5" s="380" t="s">
+      <c r="J5" s="395" t="s">
         <v>42</v>
       </c>
-      <c r="K5" s="381" t="s">
+      <c r="K5" s="396" t="s">
         <v>42</v>
       </c>
       <c r="L5" s="2"/>
@@ -6408,7 +6393,7 @@
     </row>
     <row r="6" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A6" s="281" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B6" s="250">
         <v>46073</v>
@@ -6419,8 +6404,8 @@
       <c r="D6" s="135">
         <v>1</v>
       </c>
-      <c r="E6" s="326" t="s">
-        <v>150</v>
+      <c r="E6" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F6" s="136"/>
       <c r="G6" s="137" t="s">
@@ -6430,15 +6415,15 @@
       <c r="I6" s="2"/>
       <c r="J6" s="150"/>
       <c r="K6" s="330" t="s">
-        <v>96</v>
-      </c>
-      <c r="L6" s="421"/>
-      <c r="M6" s="421"/>
-      <c r="N6" s="421"/>
-      <c r="O6" s="421"/>
-      <c r="P6" s="421"/>
-      <c r="Q6" s="421"/>
-      <c r="R6" s="421"/>
+        <v>95</v>
+      </c>
+      <c r="L6" s="428"/>
+      <c r="M6" s="428"/>
+      <c r="N6" s="428"/>
+      <c r="O6" s="428"/>
+      <c r="P6" s="428"/>
+      <c r="Q6" s="428"/>
+      <c r="R6" s="428"/>
       <c r="S6" s="2"/>
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
@@ -6534,7 +6519,7 @@
     </row>
     <row r="7" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A7" s="281" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B7" s="142" t="s">
         <v>41</v>
@@ -6545,8 +6530,8 @@
       <c r="D7" s="143">
         <v>1</v>
       </c>
-      <c r="E7" s="326" t="s">
-        <v>150</v>
+      <c r="E7" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F7" s="144"/>
       <c r="G7" s="145" t="s">
@@ -6556,7 +6541,7 @@
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
       <c r="K7" s="330" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L7" s="330"/>
       <c r="M7" s="330"/>
@@ -6671,8 +6656,8 @@
       <c r="D8" s="159">
         <v>1</v>
       </c>
-      <c r="E8" s="326" t="s">
-        <v>150</v>
+      <c r="E8" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F8" s="160"/>
       <c r="G8" s="161" t="s">
@@ -6686,13 +6671,13 @@
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
-      <c r="P8" s="425" t="s">
+      <c r="P8" s="385" t="s">
         <v>49</v>
       </c>
-      <c r="Q8" s="426" t="s">
+      <c r="Q8" s="386" t="s">
         <v>49</v>
       </c>
-      <c r="R8" s="427" t="s">
+      <c r="R8" s="387" t="s">
         <v>49</v>
       </c>
       <c r="S8" s="2"/>
@@ -6801,8 +6786,8 @@
       <c r="D9" s="164">
         <v>1</v>
       </c>
-      <c r="E9" s="326" t="s">
-        <v>150</v>
+      <c r="E9" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F9" s="165"/>
       <c r="G9" s="166" t="s">
@@ -6816,13 +6801,13 @@
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
-      <c r="P9" s="428" t="s">
+      <c r="P9" s="344" t="s">
         <v>51</v>
       </c>
-      <c r="Q9" s="429" t="s">
+      <c r="Q9" s="345" t="s">
         <v>51</v>
       </c>
-      <c r="R9" s="430" t="s">
+      <c r="R9" s="346" t="s">
         <v>51</v>
       </c>
       <c r="S9" s="2"/>
@@ -6931,8 +6916,8 @@
       <c r="D10" s="169">
         <v>1</v>
       </c>
-      <c r="E10" s="326" t="s">
-        <v>150</v>
+      <c r="E10" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F10" s="170"/>
       <c r="G10" s="171" t="s">
@@ -6946,13 +6931,13 @@
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
-      <c r="P10" s="373" t="s">
+      <c r="P10" s="388" t="s">
         <v>53</v>
       </c>
-      <c r="Q10" s="374" t="s">
+      <c r="Q10" s="389" t="s">
         <v>53</v>
       </c>
-      <c r="R10" s="375" t="s">
+      <c r="R10" s="390" t="s">
         <v>53</v>
       </c>
       <c r="S10" s="2"/>
@@ -7061,8 +7046,8 @@
       <c r="D11" s="173">
         <v>1</v>
       </c>
-      <c r="E11" s="326" t="s">
-        <v>150</v>
+      <c r="E11" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F11" s="174"/>
       <c r="G11" s="175" t="s">
@@ -7076,13 +7061,13 @@
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
-      <c r="P11" s="341" t="s">
+      <c r="P11" s="354" t="s">
         <v>56</v>
       </c>
-      <c r="Q11" s="342" t="s">
+      <c r="Q11" s="355" t="s">
         <v>56</v>
       </c>
-      <c r="R11" s="343" t="s">
+      <c r="R11" s="356" t="s">
         <v>56</v>
       </c>
       <c r="S11" s="2"/>
@@ -7191,8 +7176,8 @@
       <c r="D12" s="178">
         <v>1</v>
       </c>
-      <c r="E12" s="326" t="s">
-        <v>150</v>
+      <c r="E12" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F12" s="179"/>
       <c r="G12" s="180" t="s">
@@ -7206,13 +7191,13 @@
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
-      <c r="P12" s="344" t="s">
+      <c r="P12" s="357" t="s">
         <v>58</v>
       </c>
-      <c r="Q12" s="345" t="s">
+      <c r="Q12" s="358" t="s">
         <v>58</v>
       </c>
-      <c r="R12" s="346" t="s">
+      <c r="R12" s="359" t="s">
         <v>58</v>
       </c>
       <c r="S12" s="2"/>
@@ -7321,8 +7306,8 @@
       <c r="D13" s="183">
         <v>1</v>
       </c>
-      <c r="E13" s="326" t="s">
-        <v>150</v>
+      <c r="E13" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F13" s="184"/>
       <c r="G13" s="185" t="s">
@@ -7336,13 +7321,13 @@
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
-      <c r="P13" s="347" t="s">
+      <c r="P13" s="360" t="s">
         <v>60</v>
       </c>
-      <c r="Q13" s="348" t="s">
+      <c r="Q13" s="361" t="s">
         <v>60</v>
       </c>
-      <c r="R13" s="349" t="s">
+      <c r="R13" s="362" t="s">
         <v>60</v>
       </c>
       <c r="S13" s="2"/>
@@ -7451,8 +7436,8 @@
       <c r="D14" s="188">
         <v>1</v>
       </c>
-      <c r="E14" s="326" t="s">
-        <v>150</v>
+      <c r="E14" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="189" t="s">
@@ -7469,7 +7454,7 @@
       <c r="P14" s="190"/>
       <c r="Q14" s="191"/>
       <c r="R14" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="S14" s="281"/>
       <c r="T14" s="281"/>
@@ -7566,7 +7551,7 @@
     </row>
     <row r="15" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A15" s="281" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B15" s="192" t="s">
         <v>43</v>
@@ -7577,8 +7562,8 @@
       <c r="D15" s="194">
         <v>1</v>
       </c>
-      <c r="E15" s="326" t="s">
-        <v>149</v>
+      <c r="E15" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F15" s="195"/>
       <c r="G15" s="196" t="s">
@@ -7594,28 +7579,28 @@
       <c r="O15" s="2"/>
       <c r="P15" s="2"/>
       <c r="Q15" s="2"/>
-      <c r="R15" s="333" t="s">
-        <v>92</v>
-      </c>
-      <c r="S15" s="350" t="s">
+      <c r="R15" s="336" t="s">
+        <v>91</v>
+      </c>
+      <c r="S15" s="363" t="s">
         <v>63</v>
       </c>
-      <c r="T15" s="351" t="s">
+      <c r="T15" s="364" t="s">
         <v>63</v>
       </c>
-      <c r="U15" s="352" t="s">
+      <c r="U15" s="365" t="s">
         <v>63</v>
       </c>
-      <c r="V15" s="353" t="s">
+      <c r="V15" s="366" t="s">
         <v>63</v>
       </c>
-      <c r="W15" s="354" t="s">
+      <c r="W15" s="367" t="s">
         <v>63</v>
       </c>
-      <c r="X15" s="355" t="s">
+      <c r="X15" s="368" t="s">
         <v>63</v>
       </c>
-      <c r="Y15" s="356" t="s">
+      <c r="Y15" s="369" t="s">
         <v>63</v>
       </c>
       <c r="Z15" s="2"/>
@@ -7717,8 +7702,8 @@
       <c r="D16" s="198">
         <v>1</v>
       </c>
-      <c r="E16" s="326" t="s">
-        <v>149</v>
+      <c r="E16" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F16" s="199"/>
       <c r="G16" s="200" t="s">
@@ -7734,28 +7719,28 @@
       <c r="O16" s="2"/>
       <c r="P16" s="2"/>
       <c r="Q16" s="2"/>
-      <c r="R16" s="333" t="s">
-        <v>92</v>
-      </c>
-      <c r="S16" s="357" t="s">
+      <c r="R16" s="336" t="s">
+        <v>91</v>
+      </c>
+      <c r="S16" s="370" t="s">
         <v>65</v>
       </c>
-      <c r="T16" s="358" t="s">
+      <c r="T16" s="371" t="s">
         <v>65</v>
       </c>
-      <c r="U16" s="359" t="s">
+      <c r="U16" s="372" t="s">
         <v>65</v>
       </c>
-      <c r="V16" s="360" t="s">
+      <c r="V16" s="373" t="s">
         <v>65</v>
       </c>
-      <c r="W16" s="361" t="s">
+      <c r="W16" s="374" t="s">
         <v>65</v>
       </c>
-      <c r="X16" s="362" t="s">
+      <c r="X16" s="375" t="s">
         <v>65</v>
       </c>
-      <c r="Y16" s="363" t="s">
+      <c r="Y16" s="376" t="s">
         <v>65</v>
       </c>
       <c r="Z16" s="2"/>
@@ -7857,8 +7842,8 @@
       <c r="D17" s="202">
         <v>1</v>
       </c>
-      <c r="E17" s="326" t="s">
-        <v>149</v>
+      <c r="E17" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F17" s="203"/>
       <c r="G17" s="204" t="s">
@@ -7874,28 +7859,28 @@
       <c r="O17" s="2"/>
       <c r="P17" s="2"/>
       <c r="Q17" s="2"/>
-      <c r="R17" s="333" t="s">
+      <c r="R17" s="336" t="s">
         <v>67</v>
       </c>
-      <c r="S17" s="382" t="s">
+      <c r="S17" s="337" t="s">
         <v>67</v>
       </c>
-      <c r="T17" s="383" t="s">
+      <c r="T17" s="338" t="s">
         <v>67</v>
       </c>
-      <c r="U17" s="384" t="s">
+      <c r="U17" s="339" t="s">
         <v>67</v>
       </c>
-      <c r="V17" s="385" t="s">
+      <c r="V17" s="340" t="s">
         <v>67</v>
       </c>
-      <c r="W17" s="386" t="s">
+      <c r="W17" s="341" t="s">
         <v>67</v>
       </c>
-      <c r="X17" s="387" t="s">
+      <c r="X17" s="342" t="s">
         <v>67</v>
       </c>
-      <c r="Y17" s="388" t="s">
+      <c r="Y17" s="343" t="s">
         <v>67</v>
       </c>
       <c r="Z17" s="2"/>
@@ -7997,8 +7982,8 @@
       <c r="D18" s="207">
         <v>1</v>
       </c>
-      <c r="E18" s="326" t="s">
-        <v>149</v>
+      <c r="E18" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F18" s="208"/>
       <c r="G18" s="209" t="s">
@@ -8014,28 +7999,28 @@
       <c r="O18" s="2"/>
       <c r="P18" s="2"/>
       <c r="Q18" s="2"/>
-      <c r="R18" s="392" t="s">
+      <c r="R18" s="399" t="s">
         <v>69</v>
       </c>
-      <c r="S18" s="393" t="s">
+      <c r="S18" s="400" t="s">
         <v>69</v>
       </c>
-      <c r="T18" s="394" t="s">
+      <c r="T18" s="401" t="s">
         <v>69</v>
       </c>
-      <c r="U18" s="395" t="s">
+      <c r="U18" s="402" t="s">
         <v>69</v>
       </c>
-      <c r="V18" s="396" t="s">
+      <c r="V18" s="403" t="s">
         <v>69</v>
       </c>
-      <c r="W18" s="397" t="s">
+      <c r="W18" s="404" t="s">
         <v>69</v>
       </c>
-      <c r="X18" s="398" t="s">
+      <c r="X18" s="405" t="s">
         <v>69</v>
       </c>
-      <c r="Y18" s="399" t="s">
+      <c r="Y18" s="406" t="s">
         <v>69</v>
       </c>
       <c r="Z18" s="2"/>
@@ -8137,8 +8122,8 @@
       <c r="D19" s="147">
         <v>1</v>
       </c>
-      <c r="E19" s="326" t="s">
-        <v>149</v>
+      <c r="E19" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F19" s="148"/>
       <c r="G19" s="149" t="s">
@@ -8154,7 +8139,7 @@
       <c r="O19" s="154"/>
       <c r="P19" s="155"/>
       <c r="R19" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="S19" s="259"/>
       <c r="T19" s="259"/>
@@ -8251,7 +8236,7 @@
     </row>
     <row r="20" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A20" s="281" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B20" s="205" t="s">
         <v>43</v>
@@ -8262,8 +8247,8 @@
       <c r="D20" s="207">
         <v>1</v>
       </c>
-      <c r="E20" s="326" t="s">
-        <v>149</v>
+      <c r="E20" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F20" s="208"/>
       <c r="G20" s="209"/>
@@ -8277,16 +8262,16 @@
       <c r="O20" s="2"/>
       <c r="P20" s="2"/>
       <c r="Q20" s="2"/>
-      <c r="R20" s="407" t="s">
-        <v>95</v>
-      </c>
-      <c r="S20" s="408"/>
-      <c r="T20" s="408"/>
-      <c r="U20" s="408"/>
-      <c r="V20" s="408"/>
-      <c r="W20" s="408"/>
-      <c r="X20" s="408"/>
-      <c r="Y20" s="408"/>
+      <c r="R20" s="414" t="s">
+        <v>94</v>
+      </c>
+      <c r="S20" s="415"/>
+      <c r="T20" s="415"/>
+      <c r="U20" s="415"/>
+      <c r="V20" s="415"/>
+      <c r="W20" s="415"/>
+      <c r="X20" s="415"/>
+      <c r="Y20" s="415"/>
       <c r="Z20" s="2"/>
       <c r="AA20" s="2"/>
       <c r="AB20" s="2"/>
@@ -8386,8 +8371,8 @@
       <c r="D21" s="5">
         <v>1</v>
       </c>
-      <c r="E21" s="326" t="s">
-        <v>149</v>
+      <c r="E21" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="210" t="s">
@@ -8403,28 +8388,28 @@
       <c r="O21" s="2"/>
       <c r="P21" s="2"/>
       <c r="Q21" s="2"/>
-      <c r="R21" s="333" t="s">
+      <c r="R21" s="336" t="s">
         <v>71</v>
       </c>
-      <c r="S21" s="400" t="s">
+      <c r="S21" s="407" t="s">
         <v>71</v>
       </c>
-      <c r="T21" s="401" t="s">
+      <c r="T21" s="408" t="s">
         <v>71</v>
       </c>
-      <c r="U21" s="402" t="s">
+      <c r="U21" s="409" t="s">
         <v>71</v>
       </c>
-      <c r="V21" s="403" t="s">
+      <c r="V21" s="410" t="s">
         <v>71</v>
       </c>
-      <c r="W21" s="404" t="s">
+      <c r="W21" s="411" t="s">
         <v>71</v>
       </c>
-      <c r="X21" s="405" t="s">
+      <c r="X21" s="412" t="s">
         <v>71</v>
       </c>
-      <c r="Y21" s="406" t="s">
+      <c r="Y21" s="413" t="s">
         <v>71</v>
       </c>
       <c r="Z21" s="2"/>
@@ -8526,8 +8511,8 @@
       <c r="D22" s="139">
         <v>1</v>
       </c>
-      <c r="E22" s="326" t="s">
-        <v>149</v>
+      <c r="E22" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F22" s="140"/>
       <c r="G22" s="141" t="s">
@@ -8545,12 +8530,12 @@
       <c r="Q22" s="247"/>
       <c r="R22" s="248"/>
       <c r="S22" s="330" t="s">
-        <v>104</v>
-      </c>
-      <c r="T22" s="422"/>
-      <c r="U22" s="422"/>
-      <c r="V22" s="422"/>
-      <c r="W22" s="422"/>
+        <v>103</v>
+      </c>
+      <c r="T22" s="429"/>
+      <c r="U22" s="429"/>
+      <c r="V22" s="429"/>
+      <c r="W22" s="429"/>
       <c r="X22" s="2"/>
       <c r="Y22" s="2"/>
       <c r="Z22" s="2"/>
@@ -8652,8 +8637,8 @@
       <c r="D23" s="251">
         <v>1</v>
       </c>
-      <c r="E23" s="326" t="s">
-        <v>150</v>
+      <c r="E23" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="212" t="s">
@@ -8672,40 +8657,40 @@
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
-      <c r="U23" s="409" t="s">
+      <c r="U23" s="416" t="s">
         <v>74</v>
       </c>
-      <c r="V23" s="410" t="s">
+      <c r="V23" s="417" t="s">
         <v>74</v>
       </c>
-      <c r="W23" s="411" t="s">
+      <c r="W23" s="418" t="s">
         <v>74</v>
       </c>
-      <c r="X23" s="412" t="s">
+      <c r="X23" s="419" t="s">
         <v>74</v>
       </c>
-      <c r="Y23" s="413" t="s">
+      <c r="Y23" s="420" t="s">
         <v>74</v>
       </c>
-      <c r="Z23" s="414" t="s">
+      <c r="Z23" s="421" t="s">
         <v>74</v>
       </c>
-      <c r="AA23" s="415" t="s">
+      <c r="AA23" s="422" t="s">
         <v>74</v>
       </c>
-      <c r="AB23" s="416" t="s">
+      <c r="AB23" s="423" t="s">
         <v>74</v>
       </c>
-      <c r="AC23" s="417" t="s">
+      <c r="AC23" s="424" t="s">
         <v>74</v>
       </c>
-      <c r="AD23" s="418" t="s">
+      <c r="AD23" s="425" t="s">
         <v>74</v>
       </c>
-      <c r="AE23" s="419" t="s">
+      <c r="AE23" s="426" t="s">
         <v>74</v>
       </c>
-      <c r="AF23" s="420" t="s">
+      <c r="AF23" s="427" t="s">
         <v>74</v>
       </c>
       <c r="AG23" s="2"/>
@@ -8789,7 +8774,7 @@
     </row>
     <row r="24" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A24" s="281" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B24" s="213" t="s">
         <v>62</v>
@@ -8800,8 +8785,8 @@
       <c r="D24" s="251">
         <v>1</v>
       </c>
-      <c r="E24" s="326" t="s">
-        <v>150</v>
+      <c r="E24" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="212"/>
@@ -8823,15 +8808,15 @@
       <c r="W24" s="255"/>
       <c r="X24" s="256"/>
       <c r="Y24" s="330" t="s">
-        <v>103</v>
-      </c>
-      <c r="Z24" s="391"/>
-      <c r="AA24" s="391"/>
-      <c r="AB24" s="391"/>
-      <c r="AC24" s="391"/>
-      <c r="AD24" s="391"/>
-      <c r="AE24" s="391"/>
-      <c r="AF24" s="391"/>
+        <v>102</v>
+      </c>
+      <c r="Z24" s="398"/>
+      <c r="AA24" s="398"/>
+      <c r="AB24" s="398"/>
+      <c r="AC24" s="398"/>
+      <c r="AD24" s="398"/>
+      <c r="AE24" s="398"/>
+      <c r="AF24" s="398"/>
       <c r="AG24" s="2"/>
       <c r="AH24" s="2"/>
       <c r="AI24" s="2"/>
@@ -8913,7 +8898,7 @@
     </row>
     <row r="25" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A25" s="281" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B25" s="213" t="s">
         <v>62</v>
@@ -8924,8 +8909,8 @@
       <c r="D25" s="251">
         <v>1</v>
       </c>
-      <c r="E25" s="326" t="s">
-        <v>149</v>
+      <c r="E25" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F25" s="211"/>
       <c r="G25" s="212"/>
@@ -8947,15 +8932,15 @@
       <c r="W25" s="255"/>
       <c r="X25" s="256"/>
       <c r="Y25" s="330" t="s">
-        <v>105</v>
-      </c>
-      <c r="Z25" s="391"/>
-      <c r="AA25" s="391"/>
-      <c r="AB25" s="391"/>
-      <c r="AC25" s="391"/>
-      <c r="AD25" s="391"/>
-      <c r="AE25" s="391"/>
-      <c r="AF25" s="391"/>
+        <v>104</v>
+      </c>
+      <c r="Z25" s="398"/>
+      <c r="AA25" s="398"/>
+      <c r="AB25" s="398"/>
+      <c r="AC25" s="398"/>
+      <c r="AD25" s="398"/>
+      <c r="AE25" s="398"/>
+      <c r="AF25" s="398"/>
       <c r="AG25" s="2"/>
       <c r="AH25" s="2"/>
       <c r="AI25" s="2"/>
@@ -9037,7 +9022,7 @@
     </row>
     <row r="26" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A26" s="281" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B26" s="213" t="s">
         <v>62</v>
@@ -9048,8 +9033,8 @@
       <c r="D26" s="251">
         <v>1</v>
       </c>
-      <c r="E26" s="326" t="s">
-        <v>150</v>
+      <c r="E26" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F26" s="215"/>
       <c r="G26" s="216" t="s">
@@ -9073,15 +9058,15 @@
       <c r="W26" s="2"/>
       <c r="X26" s="2"/>
       <c r="Y26" s="330" t="s">
-        <v>108</v>
-      </c>
-      <c r="Z26" s="391"/>
-      <c r="AA26" s="391"/>
-      <c r="AB26" s="391"/>
-      <c r="AC26" s="391"/>
-      <c r="AD26" s="391"/>
-      <c r="AE26" s="391"/>
-      <c r="AF26" s="391"/>
+        <v>107</v>
+      </c>
+      <c r="Z26" s="398"/>
+      <c r="AA26" s="398"/>
+      <c r="AB26" s="398"/>
+      <c r="AC26" s="398"/>
+      <c r="AD26" s="398"/>
+      <c r="AE26" s="398"/>
+      <c r="AF26" s="398"/>
       <c r="AG26" s="2"/>
       <c r="AH26" s="2"/>
       <c r="AI26" s="2"/>
@@ -9163,7 +9148,7 @@
     </row>
     <row r="27" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A27" s="281" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B27" s="213" t="s">
         <v>62</v>
@@ -9174,8 +9159,8 @@
       <c r="D27" s="251">
         <v>1</v>
       </c>
-      <c r="E27" s="326" t="s">
-        <v>150</v>
+      <c r="E27" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F27" s="215"/>
       <c r="G27" s="216" t="s">
@@ -9198,16 +9183,16 @@
       <c r="V27" s="2"/>
       <c r="W27" s="2"/>
       <c r="X27" s="2"/>
-      <c r="AF27" s="389" t="s">
-        <v>109</v>
-      </c>
-      <c r="AG27" s="389"/>
-      <c r="AH27" s="389"/>
-      <c r="AI27" s="389"/>
-      <c r="AJ27" s="389"/>
-      <c r="AK27" s="389"/>
-      <c r="AL27" s="389"/>
-      <c r="AM27" s="389"/>
+      <c r="AF27" s="335" t="s">
+        <v>108</v>
+      </c>
+      <c r="AG27" s="335"/>
+      <c r="AH27" s="335"/>
+      <c r="AI27" s="335"/>
+      <c r="AJ27" s="335"/>
+      <c r="AK27" s="335"/>
+      <c r="AL27" s="335"/>
+      <c r="AM27" s="335"/>
       <c r="AN27" s="263"/>
       <c r="AO27" s="2"/>
       <c r="AP27" s="2"/>
@@ -9282,7 +9267,7 @@
     </row>
     <row r="28" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A28" s="281" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B28" s="214" t="s">
         <v>73</v>
@@ -9293,8 +9278,8 @@
       <c r="D28" s="251">
         <v>1</v>
       </c>
-      <c r="E28" s="326" t="s">
-        <v>150</v>
+      <c r="E28" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F28" s="215"/>
       <c r="G28" s="216"/>
@@ -9322,16 +9307,16 @@
       <c r="AC28" s="263"/>
       <c r="AD28" s="263"/>
       <c r="AE28" s="263"/>
-      <c r="AF28" s="389" t="s">
-        <v>110</v>
-      </c>
-      <c r="AG28" s="389"/>
-      <c r="AH28" s="389"/>
-      <c r="AI28" s="389"/>
-      <c r="AJ28" s="389"/>
-      <c r="AK28" s="389"/>
-      <c r="AL28" s="389"/>
-      <c r="AM28" s="389"/>
+      <c r="AF28" s="335" t="s">
+        <v>109</v>
+      </c>
+      <c r="AG28" s="335"/>
+      <c r="AH28" s="335"/>
+      <c r="AI28" s="335"/>
+      <c r="AJ28" s="335"/>
+      <c r="AK28" s="335"/>
+      <c r="AL28" s="335"/>
+      <c r="AM28" s="335"/>
       <c r="AN28" s="2"/>
       <c r="AO28" s="2"/>
       <c r="AP28" s="2"/>
@@ -9406,7 +9391,7 @@
     </row>
     <row r="29" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A29" s="281" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B29" s="214" t="s">
         <v>73</v>
@@ -9417,8 +9402,8 @@
       <c r="D29" s="251">
         <v>1</v>
       </c>
-      <c r="E29" s="326" t="s">
-        <v>150</v>
+      <c r="E29" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F29" s="215"/>
       <c r="G29" s="216"/>
@@ -9446,16 +9431,16 @@
       <c r="AC29" s="267"/>
       <c r="AD29" s="268"/>
       <c r="AE29" s="269"/>
-      <c r="AF29" s="389" t="s">
-        <v>111</v>
-      </c>
-      <c r="AG29" s="389"/>
-      <c r="AH29" s="389"/>
-      <c r="AI29" s="389"/>
-      <c r="AJ29" s="389"/>
-      <c r="AK29" s="389"/>
-      <c r="AL29" s="389"/>
-      <c r="AM29" s="389"/>
+      <c r="AF29" s="335" t="s">
+        <v>110</v>
+      </c>
+      <c r="AG29" s="335"/>
+      <c r="AH29" s="335"/>
+      <c r="AI29" s="335"/>
+      <c r="AJ29" s="335"/>
+      <c r="AK29" s="335"/>
+      <c r="AL29" s="335"/>
+      <c r="AM29" s="335"/>
       <c r="AN29" s="2"/>
       <c r="AO29" s="2"/>
       <c r="AP29" s="2"/>
@@ -9530,7 +9515,7 @@
     </row>
     <row r="30" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A30" s="281" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B30" s="214" t="s">
         <v>73</v>
@@ -9541,8 +9526,8 @@
       <c r="D30" s="251">
         <v>1</v>
       </c>
-      <c r="E30" s="326" t="s">
-        <v>149</v>
+      <c r="E30" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F30" s="215"/>
       <c r="G30" s="216"/>
@@ -9570,16 +9555,16 @@
       <c r="AC30" s="267"/>
       <c r="AD30" s="268"/>
       <c r="AE30" s="269"/>
-      <c r="AF30" s="389" t="s">
-        <v>114</v>
-      </c>
-      <c r="AG30" s="389"/>
-      <c r="AH30" s="389"/>
-      <c r="AI30" s="389"/>
-      <c r="AJ30" s="389"/>
-      <c r="AK30" s="389"/>
-      <c r="AL30" s="389"/>
-      <c r="AM30" s="389"/>
+      <c r="AF30" s="335" t="s">
+        <v>113</v>
+      </c>
+      <c r="AG30" s="335"/>
+      <c r="AH30" s="335"/>
+      <c r="AI30" s="335"/>
+      <c r="AJ30" s="335"/>
+      <c r="AK30" s="335"/>
+      <c r="AL30" s="335"/>
+      <c r="AM30" s="335"/>
       <c r="AN30" s="2"/>
       <c r="AO30" s="2"/>
       <c r="AP30" s="2"/>
@@ -9654,7 +9639,7 @@
     </row>
     <row r="31" spans="1:110" ht="17.5" customHeight="1" x14ac:dyDescent="0.8">
       <c r="A31" s="281" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B31" s="214" t="s">
         <v>73</v>
@@ -9665,8 +9650,8 @@
       <c r="D31" s="251">
         <v>1</v>
       </c>
-      <c r="E31" s="326" t="s">
-        <v>149</v>
+      <c r="E31" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F31" s="217"/>
       <c r="G31" s="218" t="s">
@@ -9696,16 +9681,16 @@
       <c r="AC31" s="2"/>
       <c r="AD31" s="272"/>
       <c r="AE31" s="273"/>
-      <c r="AF31" s="389" t="s">
-        <v>115</v>
-      </c>
-      <c r="AG31" s="389"/>
-      <c r="AH31" s="389"/>
-      <c r="AI31" s="389"/>
-      <c r="AJ31" s="389"/>
-      <c r="AK31" s="389"/>
-      <c r="AL31" s="389"/>
-      <c r="AM31" s="389"/>
+      <c r="AF31" s="335" t="s">
+        <v>114</v>
+      </c>
+      <c r="AG31" s="335"/>
+      <c r="AH31" s="335"/>
+      <c r="AI31" s="335"/>
+      <c r="AJ31" s="335"/>
+      <c r="AK31" s="335"/>
+      <c r="AL31" s="335"/>
+      <c r="AM31" s="335"/>
       <c r="AN31" s="2"/>
       <c r="AO31" s="2"/>
       <c r="AP31" s="2"/>
@@ -9780,7 +9765,7 @@
     </row>
     <row r="32" spans="1:110" ht="17.5" customHeight="1" x14ac:dyDescent="0.8">
       <c r="A32" s="281" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B32" s="214" t="s">
         <v>73</v>
@@ -9791,8 +9776,8 @@
       <c r="D32" s="251">
         <v>1</v>
       </c>
-      <c r="E32" s="326" t="s">
-        <v>149</v>
+      <c r="E32" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F32" s="217"/>
       <c r="G32" s="218" t="s">
@@ -9822,16 +9807,16 @@
       <c r="AC32" s="2"/>
       <c r="AD32" s="272"/>
       <c r="AE32" s="273"/>
-      <c r="AF32" s="389" t="s">
-        <v>117</v>
-      </c>
-      <c r="AG32" s="389"/>
-      <c r="AH32" s="389"/>
-      <c r="AI32" s="389"/>
-      <c r="AJ32" s="389"/>
-      <c r="AK32" s="389"/>
-      <c r="AL32" s="389"/>
-      <c r="AM32" s="389"/>
+      <c r="AF32" s="335" t="s">
+        <v>116</v>
+      </c>
+      <c r="AG32" s="335"/>
+      <c r="AH32" s="335"/>
+      <c r="AI32" s="335"/>
+      <c r="AJ32" s="335"/>
+      <c r="AK32" s="335"/>
+      <c r="AL32" s="335"/>
+      <c r="AM32" s="335"/>
       <c r="AN32" s="2"/>
       <c r="AO32" s="2"/>
       <c r="AP32" s="2"/>
@@ -9917,8 +9902,8 @@
       <c r="D33" s="274">
         <v>1</v>
       </c>
-      <c r="E33" s="326" t="s">
-        <v>151</v>
+      <c r="E33" s="322" t="s">
+        <v>149</v>
       </c>
       <c r="F33" s="219"/>
       <c r="G33" s="220" t="s">
@@ -9947,38 +9932,38 @@
       <c r="AB33" s="2"/>
       <c r="AC33" s="2"/>
       <c r="AD33" s="2"/>
-      <c r="AE33" s="364"/>
-      <c r="AF33" s="365" t="s">
+      <c r="AE33" s="377"/>
+      <c r="AF33" s="378" t="s">
         <v>77</v>
       </c>
-      <c r="AG33" s="366" t="s">
+      <c r="AG33" s="379" t="s">
         <v>77</v>
       </c>
-      <c r="AH33" s="367" t="s">
+      <c r="AH33" s="380" t="s">
         <v>77</v>
       </c>
-      <c r="AI33" s="368" t="s">
+      <c r="AI33" s="381" t="s">
         <v>77</v>
       </c>
-      <c r="AJ33" s="369" t="s">
+      <c r="AJ33" s="382" t="s">
         <v>77</v>
       </c>
-      <c r="AK33" s="370" t="s">
+      <c r="AK33" s="383" t="s">
         <v>77</v>
       </c>
-      <c r="AL33" s="371" t="s">
+      <c r="AL33" s="384" t="s">
         <v>77</v>
       </c>
       <c r="AM33" s="281"/>
       <c r="AN33" s="281"/>
-      <c r="AO33" s="372" t="s">
-        <v>119</v>
-      </c>
-      <c r="AP33" s="372"/>
-      <c r="AQ33" s="372"/>
-      <c r="AR33" s="372"/>
-      <c r="AS33" s="372"/>
-      <c r="AT33" s="372"/>
+      <c r="AO33" s="332" t="s">
+        <v>118</v>
+      </c>
+      <c r="AP33" s="332"/>
+      <c r="AQ33" s="332"/>
+      <c r="AR33" s="332"/>
+      <c r="AS33" s="332"/>
+      <c r="AT33" s="332"/>
       <c r="AU33" s="2"/>
       <c r="AV33" s="2"/>
       <c r="AW33" s="2"/>
@@ -10046,7 +10031,7 @@
     </row>
     <row r="34" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A34" s="281" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B34" s="221" t="s">
         <v>75</v>
@@ -10057,8 +10042,8 @@
       <c r="D34" s="278">
         <v>1</v>
       </c>
-      <c r="E34" s="326" t="s">
-        <v>151</v>
+      <c r="E34" s="322" t="s">
+        <v>149</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="224" t="s">
@@ -10095,16 +10080,16 @@
       <c r="AJ34" s="2"/>
       <c r="AK34" s="275"/>
       <c r="AL34" s="276"/>
-      <c r="AM34" s="324"/>
-      <c r="AN34" s="325"/>
-      <c r="AO34" s="372" t="s">
-        <v>128</v>
-      </c>
-      <c r="AP34" s="372"/>
-      <c r="AQ34" s="372"/>
-      <c r="AR34" s="372"/>
-      <c r="AS34" s="372"/>
-      <c r="AT34" s="372"/>
+      <c r="AM34" s="320"/>
+      <c r="AN34" s="321"/>
+      <c r="AO34" s="332" t="s">
+        <v>127</v>
+      </c>
+      <c r="AP34" s="332"/>
+      <c r="AQ34" s="332"/>
+      <c r="AR34" s="332"/>
+      <c r="AS34" s="332"/>
+      <c r="AT34" s="332"/>
       <c r="AU34" s="2"/>
       <c r="AV34" s="2"/>
       <c r="AW34" s="2"/>
@@ -10183,8 +10168,8 @@
       <c r="D35" s="278">
         <v>1</v>
       </c>
-      <c r="E35" s="326" t="s">
-        <v>150</v>
+      <c r="E35" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F35" s="223"/>
       <c r="G35" s="224"/>
@@ -10220,34 +10205,34 @@
       <c r="AK35" s="275"/>
       <c r="AL35" s="276"/>
       <c r="AM35" s="277"/>
-      <c r="AN35" s="321"/>
-      <c r="AO35" s="322"/>
-      <c r="AP35" s="322"/>
-      <c r="AQ35" s="322"/>
-      <c r="AR35" s="322"/>
-      <c r="AS35" s="322"/>
-      <c r="AT35" s="333" t="s">
-        <v>120</v>
-      </c>
-      <c r="AU35" s="334" t="s">
+      <c r="AN35" s="318"/>
+      <c r="AO35" s="319"/>
+      <c r="AP35" s="319"/>
+      <c r="AQ35" s="319"/>
+      <c r="AR35" s="319"/>
+      <c r="AS35" s="319"/>
+      <c r="AT35" s="336" t="s">
+        <v>119</v>
+      </c>
+      <c r="AU35" s="347" t="s">
         <v>81</v>
       </c>
-      <c r="AV35" s="335" t="s">
+      <c r="AV35" s="348" t="s">
         <v>81</v>
       </c>
-      <c r="AW35" s="336" t="s">
+      <c r="AW35" s="349" t="s">
         <v>81</v>
       </c>
-      <c r="AX35" s="337" t="s">
+      <c r="AX35" s="350" t="s">
         <v>81</v>
       </c>
-      <c r="AY35" s="338" t="s">
+      <c r="AY35" s="351" t="s">
         <v>81</v>
       </c>
-      <c r="AZ35" s="339" t="s">
+      <c r="AZ35" s="352" t="s">
         <v>81</v>
       </c>
-      <c r="BA35" s="340" t="s">
+      <c r="BA35" s="353" t="s">
         <v>81</v>
       </c>
       <c r="BB35" s="2"/>
@@ -10310,7 +10295,7 @@
     </row>
     <row r="36" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A36" s="281" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B36" s="225" t="s">
         <v>79</v>
@@ -10321,8 +10306,8 @@
       <c r="D36" s="278">
         <v>1</v>
       </c>
-      <c r="E36" s="326" t="s">
-        <v>150</v>
+      <c r="E36" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F36" s="227"/>
       <c r="G36" s="228"/>
@@ -10364,28 +10349,28 @@
       <c r="AQ36" s="2"/>
       <c r="AR36" s="2"/>
       <c r="AS36" s="2"/>
-      <c r="AT36" s="333" t="s">
-        <v>124</v>
-      </c>
-      <c r="AU36" s="334" t="s">
+      <c r="AT36" s="336" t="s">
+        <v>123</v>
+      </c>
+      <c r="AU36" s="347" t="s">
         <v>81</v>
       </c>
-      <c r="AV36" s="335" t="s">
+      <c r="AV36" s="348" t="s">
         <v>81</v>
       </c>
-      <c r="AW36" s="336" t="s">
+      <c r="AW36" s="349" t="s">
         <v>81</v>
       </c>
-      <c r="AX36" s="337" t="s">
+      <c r="AX36" s="350" t="s">
         <v>81</v>
       </c>
-      <c r="AY36" s="338" t="s">
+      <c r="AY36" s="351" t="s">
         <v>81</v>
       </c>
-      <c r="AZ36" s="339" t="s">
+      <c r="AZ36" s="352" t="s">
         <v>81</v>
       </c>
-      <c r="BA36" s="340" t="s">
+      <c r="BA36" s="353" t="s">
         <v>81</v>
       </c>
       <c r="BB36" s="2"/>
@@ -10448,7 +10433,7 @@
     </row>
     <row r="37" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A37" s="281" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B37" s="225" t="s">
         <v>79</v>
@@ -10459,8 +10444,8 @@
       <c r="D37" s="278">
         <v>1</v>
       </c>
-      <c r="E37" s="326" t="s">
-        <v>149</v>
+      <c r="E37" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F37" s="227"/>
       <c r="G37" s="228"/>
@@ -10502,28 +10487,28 @@
       <c r="AQ37" s="2"/>
       <c r="AR37" s="2"/>
       <c r="AS37" s="2"/>
-      <c r="AT37" s="333" t="s">
-        <v>123</v>
-      </c>
-      <c r="AU37" s="334" t="s">
+      <c r="AT37" s="336" t="s">
+        <v>122</v>
+      </c>
+      <c r="AU37" s="347" t="s">
         <v>81</v>
       </c>
-      <c r="AV37" s="335" t="s">
+      <c r="AV37" s="348" t="s">
         <v>81</v>
       </c>
-      <c r="AW37" s="336" t="s">
+      <c r="AW37" s="349" t="s">
         <v>81</v>
       </c>
-      <c r="AX37" s="337" t="s">
+      <c r="AX37" s="350" t="s">
         <v>81</v>
       </c>
-      <c r="AY37" s="338" t="s">
+      <c r="AY37" s="351" t="s">
         <v>81</v>
       </c>
-      <c r="AZ37" s="339" t="s">
+      <c r="AZ37" s="352" t="s">
         <v>81</v>
       </c>
-      <c r="BA37" s="340" t="s">
+      <c r="BA37" s="353" t="s">
         <v>81</v>
       </c>
       <c r="BB37" s="2"/>
@@ -10586,7 +10571,7 @@
     </row>
     <row r="38" spans="1:110" ht="19.5" customHeight="1" x14ac:dyDescent="0.8">
       <c r="A38" s="281" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B38" s="230" t="s">
         <v>80</v>
@@ -10597,8 +10582,8 @@
       <c r="D38" s="282">
         <v>0.75</v>
       </c>
-      <c r="E38" s="326" t="s">
-        <v>149</v>
+      <c r="E38" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F38" s="6"/>
       <c r="G38" s="229" t="s">
@@ -10650,15 +10635,15 @@
       <c r="AY38" s="2"/>
       <c r="AZ38" s="2"/>
       <c r="BA38" s="330" t="s">
-        <v>147</v>
-      </c>
-      <c r="BB38" s="432"/>
-      <c r="BC38" s="432"/>
-      <c r="BD38" s="432"/>
-      <c r="BE38" s="432"/>
-      <c r="BF38" s="432"/>
-      <c r="BG38" s="432"/>
-      <c r="BH38" s="432"/>
+        <v>146</v>
+      </c>
+      <c r="BB38" s="333"/>
+      <c r="BC38" s="333"/>
+      <c r="BD38" s="333"/>
+      <c r="BE38" s="333"/>
+      <c r="BF38" s="333"/>
+      <c r="BG38" s="333"/>
+      <c r="BH38" s="333"/>
       <c r="BI38" s="283"/>
       <c r="BJ38" s="284"/>
       <c r="BK38" s="285"/>
@@ -10712,7 +10697,7 @@
     </row>
     <row r="39" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A39" s="281" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B39" s="230" t="s">
         <v>80</v>
@@ -10723,8 +10708,8 @@
       <c r="D39" s="280">
         <v>1</v>
       </c>
-      <c r="E39" s="326" t="s">
-        <v>149</v>
+      <c r="E39" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F39" s="6"/>
       <c r="G39" s="231" t="s">
@@ -10776,15 +10761,15 @@
       <c r="AY39" s="2"/>
       <c r="AZ39" s="2"/>
       <c r="BA39" s="330" t="s">
-        <v>125</v>
-      </c>
-      <c r="BB39" s="332"/>
-      <c r="BC39" s="332"/>
-      <c r="BD39" s="332"/>
-      <c r="BE39" s="332"/>
-      <c r="BF39" s="332"/>
-      <c r="BG39" s="332"/>
-      <c r="BH39" s="332"/>
+        <v>124</v>
+      </c>
+      <c r="BB39" s="334"/>
+      <c r="BC39" s="334"/>
+      <c r="BD39" s="334"/>
+      <c r="BE39" s="334"/>
+      <c r="BF39" s="334"/>
+      <c r="BG39" s="334"/>
+      <c r="BH39" s="334"/>
       <c r="BI39" s="292"/>
       <c r="BJ39" s="293"/>
       <c r="BK39" s="294"/>
@@ -10838,7 +10823,7 @@
     </row>
     <row r="40" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A40" s="281" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B40" s="230" t="s">
         <v>80</v>
@@ -10849,8 +10834,8 @@
       <c r="D40" s="280">
         <v>1</v>
       </c>
-      <c r="E40" s="326" t="s">
-        <v>150</v>
+      <c r="E40" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F40" s="6"/>
       <c r="G40" s="231"/>
@@ -10900,7 +10885,7 @@
       <c r="AY40" s="2"/>
       <c r="AZ40" s="2"/>
       <c r="BA40" s="330" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="BB40" s="330"/>
       <c r="BC40" s="330"/>
@@ -10962,7 +10947,7 @@
     </row>
     <row r="41" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A41" s="281" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B41" s="230" t="s">
         <v>80</v>
@@ -10973,8 +10958,8 @@
       <c r="D41" s="280">
         <v>1</v>
       </c>
-      <c r="E41" s="326" t="s">
-        <v>150</v>
+      <c r="E41" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="231"/>
@@ -11024,7 +11009,7 @@
       <c r="AY41" s="2"/>
       <c r="AZ41" s="2"/>
       <c r="BA41" s="330" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="BB41" s="330"/>
       <c r="BC41" s="330"/>
@@ -11086,7 +11071,7 @@
     </row>
     <row r="42" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A42" s="281" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B42" s="230" t="s">
         <v>80</v>
@@ -11097,8 +11082,8 @@
       <c r="D42" s="280">
         <v>1</v>
       </c>
-      <c r="E42" s="326" t="s">
-        <v>150</v>
+      <c r="E42" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F42" s="6"/>
       <c r="G42" s="231"/>
@@ -11148,7 +11133,7 @@
       <c r="AY42" s="2"/>
       <c r="AZ42" s="2"/>
       <c r="BA42" s="330" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="BB42" s="330"/>
       <c r="BC42" s="330"/>
@@ -11210,7 +11195,7 @@
     </row>
     <row r="43" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A43" s="281" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B43" s="230" t="s">
         <v>80</v>
@@ -11221,8 +11206,8 @@
       <c r="D43" s="280">
         <v>1</v>
       </c>
-      <c r="E43" s="326" t="s">
-        <v>150</v>
+      <c r="E43" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F43" s="6"/>
       <c r="G43" s="231"/>
@@ -11272,7 +11257,7 @@
       <c r="AY43" s="2"/>
       <c r="AZ43" s="2"/>
       <c r="BA43" s="330" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="BB43" s="330"/>
       <c r="BC43" s="330"/>
@@ -11334,7 +11319,7 @@
     </row>
     <row r="44" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A44" s="281" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B44" s="230" t="s">
         <v>80</v>
@@ -11345,8 +11330,8 @@
       <c r="D44" s="280">
         <v>1</v>
       </c>
-      <c r="E44" s="326" t="s">
-        <v>149</v>
+      <c r="E44" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F44" s="6"/>
       <c r="G44" s="231"/>
@@ -11396,7 +11381,7 @@
       <c r="AY44" s="2"/>
       <c r="AZ44" s="2"/>
       <c r="BA44" s="330" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="BB44" s="330"/>
       <c r="BC44" s="330"/>
@@ -11458,7 +11443,7 @@
     </row>
     <row r="45" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A45" s="281" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B45" s="230" t="s">
         <v>80</v>
@@ -11469,8 +11454,8 @@
       <c r="D45" s="280">
         <v>1</v>
       </c>
-      <c r="E45" s="326" t="s">
-        <v>150</v>
+      <c r="E45" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F45" s="6"/>
       <c r="G45" s="231"/>
@@ -11520,7 +11505,7 @@
       <c r="AY45" s="2"/>
       <c r="AZ45" s="2"/>
       <c r="BA45" s="330" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="BB45" s="330"/>
       <c r="BC45" s="330"/>
@@ -11582,7 +11567,7 @@
     </row>
     <row r="46" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A46" s="281" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B46" s="230" t="s">
         <v>80</v>
@@ -11593,8 +11578,8 @@
       <c r="D46" s="280">
         <v>1</v>
       </c>
-      <c r="E46" s="326" t="s">
-        <v>149</v>
+      <c r="E46" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F46" s="6"/>
       <c r="G46" s="231"/>
@@ -11644,7 +11629,7 @@
       <c r="AY46" s="2"/>
       <c r="AZ46" s="2"/>
       <c r="BA46" s="330" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="BB46" s="330"/>
       <c r="BC46" s="330"/>
@@ -11706,7 +11691,7 @@
     </row>
     <row r="47" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A47" s="281" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B47" s="230" t="s">
         <v>80</v>
@@ -11717,8 +11702,8 @@
       <c r="D47" s="280">
         <v>1</v>
       </c>
-      <c r="E47" s="326" t="s">
-        <v>150</v>
+      <c r="E47" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F47" s="6"/>
       <c r="G47" s="231"/>
@@ -11768,7 +11753,7 @@
       <c r="AY47" s="2"/>
       <c r="AZ47" s="2"/>
       <c r="BA47" s="330" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="BB47" s="330"/>
       <c r="BC47" s="330"/>
@@ -11830,7 +11815,7 @@
     </row>
     <row r="48" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A48" s="281" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B48" s="230" t="s">
         <v>80</v>
@@ -11841,8 +11826,8 @@
       <c r="D48" s="280">
         <v>1</v>
       </c>
-      <c r="E48" s="326" t="s">
-        <v>150</v>
+      <c r="E48" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F48" s="6"/>
       <c r="G48" s="231"/>
@@ -11892,7 +11877,7 @@
       <c r="AY48" s="2"/>
       <c r="AZ48" s="2"/>
       <c r="BA48" s="330" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="BB48" s="330"/>
       <c r="BC48" s="330"/>
@@ -11954,7 +11939,7 @@
     </row>
     <row r="49" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A49" s="281" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B49" s="230" t="s">
         <v>80</v>
@@ -11965,8 +11950,8 @@
       <c r="D49" s="280">
         <v>1</v>
       </c>
-      <c r="E49" s="326" t="s">
-        <v>149</v>
+      <c r="E49" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F49" s="6"/>
       <c r="G49" s="231"/>
@@ -12016,7 +12001,7 @@
       <c r="AY49" s="2"/>
       <c r="AZ49" s="2"/>
       <c r="BA49" s="330" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="BB49" s="330"/>
       <c r="BC49" s="330"/>
@@ -12078,7 +12063,7 @@
     </row>
     <row r="50" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A50" s="281" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B50" s="230" t="s">
         <v>80</v>
@@ -12089,8 +12074,8 @@
       <c r="D50" s="280">
         <v>1</v>
       </c>
-      <c r="E50" s="326" t="s">
-        <v>150</v>
+      <c r="E50" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F50" s="6"/>
       <c r="G50" s="231"/>
@@ -12140,7 +12125,7 @@
       <c r="AY50" s="2"/>
       <c r="AZ50" s="2"/>
       <c r="BA50" s="330" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="BB50" s="330"/>
       <c r="BC50" s="330"/>
@@ -12202,7 +12187,7 @@
     </row>
     <row r="51" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A51" s="281" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B51" s="230" t="s">
         <v>80</v>
@@ -12213,8 +12198,8 @@
       <c r="D51" s="280">
         <v>1</v>
       </c>
-      <c r="E51" s="326" t="s">
-        <v>149</v>
+      <c r="E51" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F51" s="6"/>
       <c r="G51" s="231"/>
@@ -12264,7 +12249,7 @@
       <c r="AY51" s="2"/>
       <c r="AZ51" s="2"/>
       <c r="BA51" s="330" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="BB51" s="330"/>
       <c r="BC51" s="330"/>
@@ -12326,7 +12311,7 @@
     </row>
     <row r="52" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A52" s="281" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B52" s="230" t="s">
         <v>80</v>
@@ -12337,8 +12322,8 @@
       <c r="D52" s="280">
         <v>1</v>
       </c>
-      <c r="E52" s="326" t="s">
-        <v>149</v>
+      <c r="E52" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F52" s="6"/>
       <c r="G52" s="231"/>
@@ -12388,7 +12373,7 @@
       <c r="AY52" s="2"/>
       <c r="AZ52" s="2"/>
       <c r="BA52" s="330" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="BB52" s="330"/>
       <c r="BC52" s="330"/>
@@ -12450,7 +12435,7 @@
     </row>
     <row r="53" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A53" s="281" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B53" s="230" t="s">
         <v>80</v>
@@ -12461,8 +12446,8 @@
       <c r="D53" s="280">
         <v>1</v>
       </c>
-      <c r="E53" s="326" t="s">
-        <v>150</v>
+      <c r="E53" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F53" s="6"/>
       <c r="G53" s="231"/>
@@ -12512,7 +12497,7 @@
       <c r="AY53" s="2"/>
       <c r="AZ53" s="2"/>
       <c r="BA53" s="330" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="BB53" s="330"/>
       <c r="BC53" s="330"/>
@@ -12574,7 +12559,7 @@
     </row>
     <row r="54" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A54" s="281" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B54" s="230" t="s">
         <v>80</v>
@@ -12585,8 +12570,8 @@
       <c r="D54" s="280">
         <v>1</v>
       </c>
-      <c r="E54" s="326" t="s">
-        <v>150</v>
+      <c r="E54" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F54" s="6"/>
       <c r="G54" s="231"/>
@@ -12636,7 +12621,7 @@
       <c r="AY54" s="2"/>
       <c r="AZ54" s="2"/>
       <c r="BA54" s="330" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="BB54" s="330"/>
       <c r="BC54" s="330"/>
@@ -12698,7 +12683,7 @@
     </row>
     <row r="55" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A55" s="281" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B55" s="230" t="s">
         <v>80</v>
@@ -12709,8 +12694,8 @@
       <c r="D55" s="280">
         <v>1</v>
       </c>
-      <c r="E55" s="326" t="s">
-        <v>151</v>
+      <c r="E55" s="322" t="s">
+        <v>149</v>
       </c>
       <c r="F55" s="6"/>
       <c r="G55" s="231"/>
@@ -12760,7 +12745,7 @@
       <c r="AY55" s="2"/>
       <c r="AZ55" s="2"/>
       <c r="BA55" s="330" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="BB55" s="330"/>
       <c r="BC55" s="330"/>
@@ -12822,7 +12807,7 @@
     </row>
     <row r="56" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A56" s="281" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B56" s="230" t="s">
         <v>80</v>
@@ -12833,8 +12818,8 @@
       <c r="D56" s="280">
         <v>1</v>
       </c>
-      <c r="E56" s="326" t="s">
-        <v>150</v>
+      <c r="E56" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F56" s="6"/>
       <c r="G56" s="231"/>
@@ -12884,7 +12869,7 @@
       <c r="AY56" s="2"/>
       <c r="AZ56" s="2"/>
       <c r="BA56" s="330" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="BB56" s="330"/>
       <c r="BC56" s="330"/>
@@ -12946,7 +12931,7 @@
     </row>
     <row r="57" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A57" s="281" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B57" s="290">
         <v>46122</v>
@@ -12957,8 +12942,8 @@
       <c r="D57" s="280">
         <v>1</v>
       </c>
-      <c r="E57" s="326" t="s">
-        <v>150</v>
+      <c r="E57" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F57" s="6"/>
       <c r="G57" s="231"/>
@@ -13007,24 +12992,24 @@
       <c r="AX57" s="2"/>
       <c r="AY57" s="2"/>
       <c r="AZ57" s="2"/>
-      <c r="BA57" s="327"/>
-      <c r="BB57" s="327"/>
-      <c r="BC57" s="327"/>
-      <c r="BD57" s="327"/>
-      <c r="BE57" s="327"/>
-      <c r="BF57" s="327"/>
-      <c r="BG57" s="327"/>
+      <c r="BA57" s="323"/>
+      <c r="BB57" s="323"/>
+      <c r="BC57" s="323"/>
+      <c r="BD57" s="323"/>
+      <c r="BE57" s="323"/>
+      <c r="BF57" s="323"/>
+      <c r="BG57" s="323"/>
       <c r="BH57" s="330" t="s">
-        <v>175</v>
-      </c>
-      <c r="BI57" s="433"/>
-      <c r="BJ57" s="433"/>
-      <c r="BK57" s="433"/>
-      <c r="BL57" s="433"/>
-      <c r="BM57" s="433"/>
-      <c r="BN57" s="433"/>
-      <c r="BO57" s="433"/>
-      <c r="BP57" s="328"/>
+        <v>171</v>
+      </c>
+      <c r="BI57" s="331"/>
+      <c r="BJ57" s="331"/>
+      <c r="BK57" s="331"/>
+      <c r="BL57" s="331"/>
+      <c r="BM57" s="331"/>
+      <c r="BN57" s="331"/>
+      <c r="BO57" s="331"/>
+      <c r="BP57" s="324"/>
       <c r="BQ57" s="2"/>
       <c r="BR57" s="2"/>
       <c r="BS57" s="2"/>
@@ -13070,7 +13055,7 @@
     </row>
     <row r="58" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A58" s="281" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B58" s="290">
         <v>46122</v>
@@ -13081,8 +13066,8 @@
       <c r="D58" s="280">
         <v>1</v>
       </c>
-      <c r="E58" s="326" t="s">
-        <v>150</v>
+      <c r="E58" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F58" s="6"/>
       <c r="G58" s="231"/>
@@ -13131,23 +13116,23 @@
       <c r="AX58" s="2"/>
       <c r="AY58" s="2"/>
       <c r="AZ58" s="2"/>
-      <c r="BA58" s="327"/>
-      <c r="BB58" s="327"/>
-      <c r="BC58" s="327"/>
-      <c r="BD58" s="327"/>
-      <c r="BE58" s="327"/>
-      <c r="BF58" s="327"/>
-      <c r="BG58" s="327"/>
+      <c r="BA58" s="323"/>
+      <c r="BB58" s="323"/>
+      <c r="BC58" s="323"/>
+      <c r="BD58" s="323"/>
+      <c r="BE58" s="323"/>
+      <c r="BF58" s="323"/>
+      <c r="BG58" s="323"/>
       <c r="BH58" s="330" t="s">
-        <v>176</v>
-      </c>
-      <c r="BI58" s="433"/>
-      <c r="BJ58" s="433"/>
-      <c r="BK58" s="433"/>
-      <c r="BL58" s="433"/>
-      <c r="BM58" s="433"/>
-      <c r="BN58" s="433"/>
-      <c r="BO58" s="433"/>
+        <v>172</v>
+      </c>
+      <c r="BI58" s="331"/>
+      <c r="BJ58" s="331"/>
+      <c r="BK58" s="331"/>
+      <c r="BL58" s="331"/>
+      <c r="BM58" s="331"/>
+      <c r="BN58" s="331"/>
+      <c r="BO58" s="331"/>
       <c r="BP58" s="2"/>
       <c r="BQ58" s="2"/>
       <c r="BR58" s="2"/>
@@ -13194,7 +13179,7 @@
     </row>
     <row r="59" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A59" s="281" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="B59" s="290">
         <v>46122</v>
@@ -13205,8 +13190,8 @@
       <c r="D59" s="280">
         <v>1</v>
       </c>
-      <c r="E59" s="326" t="s">
-        <v>150</v>
+      <c r="E59" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F59" s="6"/>
       <c r="G59" s="231"/>
@@ -13255,23 +13240,23 @@
       <c r="AX59" s="2"/>
       <c r="AY59" s="2"/>
       <c r="AZ59" s="2"/>
-      <c r="BA59" s="327"/>
-      <c r="BB59" s="327"/>
-      <c r="BC59" s="327"/>
-      <c r="BD59" s="327"/>
-      <c r="BE59" s="327"/>
-      <c r="BF59" s="327"/>
-      <c r="BG59" s="327"/>
+      <c r="BA59" s="323"/>
+      <c r="BB59" s="323"/>
+      <c r="BC59" s="323"/>
+      <c r="BD59" s="323"/>
+      <c r="BE59" s="323"/>
+      <c r="BF59" s="323"/>
+      <c r="BG59" s="323"/>
       <c r="BH59" s="330" t="s">
-        <v>177</v>
-      </c>
-      <c r="BI59" s="433"/>
-      <c r="BJ59" s="433"/>
-      <c r="BK59" s="433"/>
-      <c r="BL59" s="433"/>
-      <c r="BM59" s="433"/>
-      <c r="BN59" s="433"/>
-      <c r="BO59" s="433"/>
+        <v>173</v>
+      </c>
+      <c r="BI59" s="331"/>
+      <c r="BJ59" s="331"/>
+      <c r="BK59" s="331"/>
+      <c r="BL59" s="331"/>
+      <c r="BM59" s="331"/>
+      <c r="BN59" s="331"/>
+      <c r="BO59" s="331"/>
       <c r="BP59" s="2"/>
       <c r="BQ59" s="2"/>
       <c r="BR59" s="2"/>
@@ -13318,7 +13303,7 @@
     </row>
     <row r="60" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A60" s="281" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="B60" s="290">
         <v>46122</v>
@@ -13329,8 +13314,8 @@
       <c r="D60" s="280">
         <v>1</v>
       </c>
-      <c r="E60" s="326" t="s">
-        <v>182</v>
+      <c r="E60" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F60" s="6"/>
       <c r="G60" s="231"/>
@@ -13379,23 +13364,23 @@
       <c r="AX60" s="2"/>
       <c r="AY60" s="2"/>
       <c r="AZ60" s="2"/>
-      <c r="BA60" s="327"/>
-      <c r="BB60" s="327"/>
-      <c r="BC60" s="327"/>
-      <c r="BD60" s="327"/>
-      <c r="BE60" s="327"/>
-      <c r="BF60" s="327"/>
-      <c r="BG60" s="327"/>
+      <c r="BA60" s="323"/>
+      <c r="BB60" s="323"/>
+      <c r="BC60" s="323"/>
+      <c r="BD60" s="323"/>
+      <c r="BE60" s="323"/>
+      <c r="BF60" s="323"/>
+      <c r="BG60" s="323"/>
       <c r="BH60" s="330" t="s">
-        <v>178</v>
-      </c>
-      <c r="BI60" s="433"/>
-      <c r="BJ60" s="433"/>
-      <c r="BK60" s="433"/>
-      <c r="BL60" s="433"/>
-      <c r="BM60" s="433"/>
-      <c r="BN60" s="433"/>
-      <c r="BO60" s="433"/>
+        <v>174</v>
+      </c>
+      <c r="BI60" s="331"/>
+      <c r="BJ60" s="331"/>
+      <c r="BK60" s="331"/>
+      <c r="BL60" s="331"/>
+      <c r="BM60" s="331"/>
+      <c r="BN60" s="331"/>
+      <c r="BO60" s="331"/>
       <c r="BP60" s="2"/>
       <c r="BQ60" s="2"/>
       <c r="BR60" s="2"/>
@@ -13441,8 +13426,8 @@
       <c r="DF60" s="2"/>
     </row>
     <row r="61" spans="1:110" ht="53.25" customHeight="1" x14ac:dyDescent="0.8">
-      <c r="A61" s="323" t="s">
-        <v>172</v>
+      <c r="A61" s="281" t="s">
+        <v>170</v>
       </c>
       <c r="B61" s="290">
         <v>46122</v>
@@ -13451,12 +13436,12 @@
         <v>83</v>
       </c>
       <c r="D61" s="280">
-        <v>0.95</v>
-      </c>
-      <c r="E61" s="326"/>
-      <c r="F61" s="6" t="s">
-        <v>173</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E61" s="322" t="s">
+        <v>149</v>
+      </c>
+      <c r="F61" s="6"/>
       <c r="G61" s="231"/>
       <c r="H61" s="2"/>
       <c r="I61" s="2"/>
@@ -13503,23 +13488,23 @@
       <c r="AX61" s="2"/>
       <c r="AY61" s="2"/>
       <c r="AZ61" s="2"/>
-      <c r="BA61" s="327"/>
-      <c r="BB61" s="327"/>
-      <c r="BC61" s="327"/>
-      <c r="BD61" s="327"/>
-      <c r="BE61" s="327"/>
-      <c r="BF61" s="327"/>
-      <c r="BG61" s="327"/>
-      <c r="BH61" s="331" t="s">
-        <v>179</v>
-      </c>
-      <c r="BI61" s="436"/>
-      <c r="BJ61" s="436"/>
-      <c r="BK61" s="436"/>
-      <c r="BL61" s="436"/>
-      <c r="BM61" s="436"/>
-      <c r="BN61" s="436"/>
-      <c r="BO61" s="436"/>
+      <c r="BA61" s="323"/>
+      <c r="BB61" s="323"/>
+      <c r="BC61" s="323"/>
+      <c r="BD61" s="323"/>
+      <c r="BE61" s="323"/>
+      <c r="BF61" s="323"/>
+      <c r="BG61" s="323"/>
+      <c r="BH61" s="330" t="s">
+        <v>175</v>
+      </c>
+      <c r="BI61" s="331"/>
+      <c r="BJ61" s="331"/>
+      <c r="BK61" s="331"/>
+      <c r="BL61" s="331"/>
+      <c r="BM61" s="331"/>
+      <c r="BN61" s="331"/>
+      <c r="BO61" s="331"/>
       <c r="BP61" s="2"/>
       <c r="BQ61" s="2"/>
       <c r="BR61" s="2"/>
@@ -13577,8 +13562,8 @@
       <c r="D62" s="280">
         <v>1</v>
       </c>
-      <c r="E62" s="326" t="s">
-        <v>151</v>
+      <c r="E62" s="322" t="s">
+        <v>149</v>
       </c>
       <c r="F62" s="6"/>
       <c r="G62" s="231"/>
@@ -13627,15 +13612,15 @@
       <c r="AX62" s="2"/>
       <c r="AY62" s="2"/>
       <c r="AZ62" s="2"/>
-      <c r="BA62" s="327"/>
-      <c r="BB62" s="327"/>
-      <c r="BC62" s="327"/>
-      <c r="BD62" s="327"/>
-      <c r="BE62" s="327"/>
-      <c r="BF62" s="327"/>
-      <c r="BG62" s="327"/>
+      <c r="BA62" s="323"/>
+      <c r="BB62" s="323"/>
+      <c r="BC62" s="323"/>
+      <c r="BD62" s="323"/>
+      <c r="BE62" s="323"/>
+      <c r="BF62" s="323"/>
+      <c r="BG62" s="323"/>
       <c r="BH62" s="330" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="BI62" s="330"/>
       <c r="BJ62" s="330"/>
@@ -13690,7 +13675,7 @@
     </row>
     <row r="63" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A63" s="281" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="B63" s="290">
         <v>46122</v>
@@ -13701,8 +13686,8 @@
       <c r="D63" s="280">
         <v>1</v>
       </c>
-      <c r="E63" s="326" t="s">
-        <v>150</v>
+      <c r="E63" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F63" s="6"/>
       <c r="G63" s="231"/>
@@ -13751,15 +13736,15 @@
       <c r="AX63" s="2"/>
       <c r="AY63" s="2"/>
       <c r="AZ63" s="2"/>
-      <c r="BA63" s="327"/>
-      <c r="BB63" s="327"/>
-      <c r="BC63" s="327"/>
-      <c r="BD63" s="327"/>
-      <c r="BE63" s="327"/>
-      <c r="BF63" s="327"/>
-      <c r="BG63" s="327"/>
+      <c r="BA63" s="323"/>
+      <c r="BB63" s="323"/>
+      <c r="BC63" s="323"/>
+      <c r="BD63" s="323"/>
+      <c r="BE63" s="323"/>
+      <c r="BF63" s="323"/>
+      <c r="BG63" s="323"/>
       <c r="BH63" s="330" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="BI63" s="330"/>
       <c r="BJ63" s="330"/>
@@ -13814,7 +13799,7 @@
     </row>
     <row r="64" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A64" s="281" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B64" s="290">
         <v>46122</v>
@@ -13825,8 +13810,8 @@
       <c r="D64" s="280">
         <v>1</v>
       </c>
-      <c r="E64" s="326" t="s">
-        <v>150</v>
+      <c r="E64" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F64" s="6"/>
       <c r="G64" s="231"/>
@@ -13875,15 +13860,15 @@
       <c r="AX64" s="2"/>
       <c r="AY64" s="2"/>
       <c r="AZ64" s="2"/>
-      <c r="BA64" s="327"/>
-      <c r="BB64" s="327"/>
-      <c r="BC64" s="327"/>
-      <c r="BD64" s="327"/>
-      <c r="BE64" s="327"/>
-      <c r="BF64" s="327"/>
-      <c r="BG64" s="327"/>
+      <c r="BA64" s="323"/>
+      <c r="BB64" s="323"/>
+      <c r="BC64" s="323"/>
+      <c r="BD64" s="323"/>
+      <c r="BE64" s="323"/>
+      <c r="BF64" s="323"/>
+      <c r="BG64" s="323"/>
       <c r="BH64" s="330" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="BI64" s="330"/>
       <c r="BJ64" s="330"/>
@@ -13938,7 +13923,7 @@
     </row>
     <row r="65" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A65" s="281" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="B65" s="290">
         <v>46122</v>
@@ -13949,8 +13934,8 @@
       <c r="D65" s="280">
         <v>1</v>
       </c>
-      <c r="E65" s="326" t="s">
-        <v>150</v>
+      <c r="E65" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F65" s="6"/>
       <c r="G65" s="231"/>
@@ -13999,15 +13984,15 @@
       <c r="AX65" s="2"/>
       <c r="AY65" s="2"/>
       <c r="AZ65" s="2"/>
-      <c r="BA65" s="327"/>
-      <c r="BB65" s="327"/>
-      <c r="BC65" s="327"/>
-      <c r="BD65" s="327"/>
-      <c r="BE65" s="327"/>
-      <c r="BF65" s="327"/>
-      <c r="BG65" s="327"/>
+      <c r="BA65" s="323"/>
+      <c r="BB65" s="323"/>
+      <c r="BC65" s="323"/>
+      <c r="BD65" s="323"/>
+      <c r="BE65" s="323"/>
+      <c r="BF65" s="323"/>
+      <c r="BG65" s="323"/>
       <c r="BH65" s="330" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="BI65" s="330"/>
       <c r="BJ65" s="330"/>
@@ -14062,7 +14047,7 @@
     </row>
     <row r="66" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A66" s="281" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="B66" s="290">
         <v>46122</v>
@@ -14073,8 +14058,8 @@
       <c r="D66" s="280">
         <v>1</v>
       </c>
-      <c r="E66" s="326" t="s">
-        <v>150</v>
+      <c r="E66" s="322" t="s">
+        <v>148</v>
       </c>
       <c r="F66" s="6"/>
       <c r="G66" s="231"/>
@@ -14123,15 +14108,15 @@
       <c r="AX66" s="2"/>
       <c r="AY66" s="2"/>
       <c r="AZ66" s="2"/>
-      <c r="BA66" s="327"/>
-      <c r="BB66" s="327"/>
-      <c r="BC66" s="327"/>
-      <c r="BD66" s="327"/>
-      <c r="BE66" s="327"/>
-      <c r="BF66" s="327"/>
-      <c r="BG66" s="327"/>
+      <c r="BA66" s="323"/>
+      <c r="BB66" s="323"/>
+      <c r="BC66" s="323"/>
+      <c r="BD66" s="323"/>
+      <c r="BE66" s="323"/>
+      <c r="BF66" s="323"/>
+      <c r="BG66" s="323"/>
       <c r="BH66" s="330" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="BI66" s="330"/>
       <c r="BJ66" s="330"/>
@@ -14186,7 +14171,7 @@
     </row>
     <row r="67" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A67" s="281" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="B67" s="290">
         <v>46122</v>
@@ -14197,8 +14182,8 @@
       <c r="D67" s="280">
         <v>1</v>
       </c>
-      <c r="E67" s="326" t="s">
-        <v>182</v>
+      <c r="E67" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F67" s="6"/>
       <c r="G67" s="231"/>
@@ -14247,15 +14232,15 @@
       <c r="AX67" s="2"/>
       <c r="AY67" s="2"/>
       <c r="AZ67" s="2"/>
-      <c r="BA67" s="327"/>
-      <c r="BB67" s="327"/>
-      <c r="BC67" s="327"/>
-      <c r="BD67" s="327"/>
-      <c r="BE67" s="327"/>
-      <c r="BF67" s="327"/>
-      <c r="BG67" s="327"/>
+      <c r="BA67" s="323"/>
+      <c r="BB67" s="323"/>
+      <c r="BC67" s="323"/>
+      <c r="BD67" s="323"/>
+      <c r="BE67" s="323"/>
+      <c r="BF67" s="323"/>
+      <c r="BG67" s="323"/>
       <c r="BH67" s="330" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="BI67" s="330"/>
       <c r="BJ67" s="330"/>
@@ -14310,7 +14295,7 @@
     </row>
     <row r="68" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A68" s="281" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="B68" s="290">
         <v>46122</v>
@@ -14321,8 +14306,8 @@
       <c r="D68" s="280">
         <v>1</v>
       </c>
-      <c r="E68" s="326" t="s">
-        <v>182</v>
+      <c r="E68" s="322" t="s">
+        <v>177</v>
       </c>
       <c r="F68" s="6"/>
       <c r="G68" s="231"/>
@@ -14371,15 +14356,15 @@
       <c r="AX68" s="2"/>
       <c r="AY68" s="2"/>
       <c r="AZ68" s="2"/>
-      <c r="BA68" s="327"/>
-      <c r="BB68" s="327"/>
-      <c r="BC68" s="327"/>
-      <c r="BD68" s="327"/>
-      <c r="BE68" s="327"/>
-      <c r="BF68" s="327"/>
-      <c r="BG68" s="327"/>
+      <c r="BA68" s="323"/>
+      <c r="BB68" s="323"/>
+      <c r="BC68" s="323"/>
+      <c r="BD68" s="323"/>
+      <c r="BE68" s="323"/>
+      <c r="BF68" s="323"/>
+      <c r="BG68" s="323"/>
       <c r="BH68" s="330" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="BI68" s="330"/>
       <c r="BJ68" s="330"/>
@@ -14434,7 +14419,7 @@
     </row>
     <row r="69" spans="1:110" x14ac:dyDescent="0.8">
       <c r="A69" s="281" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B69" s="290">
         <v>46122</v>
@@ -14442,11 +14427,11 @@
       <c r="C69" s="232" t="s">
         <v>83</v>
       </c>
-      <c r="D69" s="326">
+      <c r="D69" s="322">
         <v>1</v>
       </c>
-      <c r="E69" s="435" t="s">
-        <v>151</v>
+      <c r="E69" s="326" t="s">
+        <v>149</v>
       </c>
       <c r="F69" s="233"/>
       <c r="G69" s="234" t="s">
@@ -14505,15 +14490,15 @@
       <c r="BF69" s="303"/>
       <c r="BG69" s="304"/>
       <c r="BH69" s="330" t="s">
-        <v>180</v>
-      </c>
-      <c r="BI69" s="433"/>
-      <c r="BJ69" s="433"/>
-      <c r="BK69" s="433"/>
-      <c r="BL69" s="433"/>
-      <c r="BM69" s="433"/>
-      <c r="BN69" s="433"/>
-      <c r="BO69" s="433"/>
+        <v>176</v>
+      </c>
+      <c r="BI69" s="331"/>
+      <c r="BJ69" s="331"/>
+      <c r="BK69" s="331"/>
+      <c r="BL69" s="331"/>
+      <c r="BM69" s="331"/>
+      <c r="BN69" s="331"/>
+      <c r="BO69" s="331"/>
       <c r="BP69" s="2"/>
       <c r="BQ69" s="2"/>
       <c r="BR69" s="2"/>
@@ -14559,17 +14544,21 @@
       <c r="DF69" s="2"/>
     </row>
     <row r="70" spans="1:110" x14ac:dyDescent="0.8">
-      <c r="A70" s="2" t="s">
-        <v>84</v>
+      <c r="A70" s="281" t="s">
+        <v>207</v>
       </c>
       <c r="B70" s="291">
         <v>46129</v>
       </c>
-      <c r="C70" s="431">
+      <c r="C70" s="325">
         <v>46134</v>
       </c>
-      <c r="D70" s="235"/>
-      <c r="E70" s="235"/>
+      <c r="D70" s="327">
+        <v>1</v>
+      </c>
+      <c r="E70" s="326" t="s">
+        <v>149</v>
+      </c>
       <c r="F70" s="236"/>
       <c r="G70" s="237" t="s">
         <v>0</v>
@@ -14633,15 +14622,15 @@
       <c r="BL70" s="312"/>
       <c r="BM70" s="313"/>
       <c r="BN70" s="2"/>
-      <c r="BO70" s="329" t="s">
-        <v>195</v>
-      </c>
-      <c r="BP70" s="329"/>
-      <c r="BQ70" s="329"/>
-      <c r="BR70" s="329"/>
-      <c r="BS70" s="329"/>
-      <c r="BT70" s="434"/>
-      <c r="BU70" s="434"/>
+      <c r="BO70" s="332" t="s">
+        <v>208</v>
+      </c>
+      <c r="BP70" s="332"/>
+      <c r="BQ70" s="332"/>
+      <c r="BR70" s="332"/>
+      <c r="BS70" s="332"/>
+      <c r="BT70" s="2"/>
+      <c r="BU70" s="2"/>
       <c r="BV70" s="2"/>
       <c r="BW70" s="2"/>
       <c r="BX70" s="2"/>
@@ -14680,19 +14669,25 @@
       <c r="DE70" s="2"/>
       <c r="DF70" s="2"/>
     </row>
-    <row r="71" spans="1:110" x14ac:dyDescent="0.8">
-      <c r="A71" s="2" t="s">
-        <v>209</v>
+    <row r="71" spans="1:110" ht="48" x14ac:dyDescent="0.8">
+      <c r="A71" s="328" t="s">
+        <v>203</v>
       </c>
       <c r="B71" s="291">
         <v>46129</v>
       </c>
       <c r="C71" s="235" t="s">
-        <v>85</v>
-      </c>
-      <c r="D71" s="235"/>
-      <c r="E71" s="235"/>
-      <c r="F71" s="236"/>
+        <v>84</v>
+      </c>
+      <c r="D71" s="327">
+        <v>0</v>
+      </c>
+      <c r="E71" s="326" t="s">
+        <v>177</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>206</v>
+      </c>
       <c r="G71" s="237"/>
       <c r="H71" s="2"/>
       <c r="I71" s="2"/>
@@ -14753,15 +14748,15 @@
       <c r="BL71" s="312"/>
       <c r="BM71" s="313"/>
       <c r="BN71" s="2"/>
-      <c r="BO71" s="329" t="s">
-        <v>203</v>
-      </c>
-      <c r="BP71" s="329"/>
-      <c r="BQ71" s="329"/>
-      <c r="BR71" s="329"/>
-      <c r="BS71" s="329"/>
-      <c r="BT71" s="329"/>
-      <c r="BU71" s="329"/>
+      <c r="BO71" s="434" t="s">
+        <v>197</v>
+      </c>
+      <c r="BP71" s="434"/>
+      <c r="BQ71" s="434"/>
+      <c r="BR71" s="434"/>
+      <c r="BS71" s="434"/>
+      <c r="BT71" s="434"/>
+      <c r="BU71" s="434"/>
       <c r="BV71" s="2"/>
       <c r="BW71" s="2"/>
       <c r="BX71" s="2"/>
@@ -14801,17 +14796,21 @@
       <c r="DF71" s="2"/>
     </row>
     <row r="72" spans="1:110" x14ac:dyDescent="0.8">
-      <c r="A72" s="2" t="s">
-        <v>204</v>
+      <c r="A72" s="281" t="s">
+        <v>198</v>
       </c>
       <c r="B72" s="291">
         <v>46129</v>
       </c>
       <c r="C72" s="235" t="s">
-        <v>85</v>
-      </c>
-      <c r="D72" s="235"/>
-      <c r="E72" s="235"/>
+        <v>84</v>
+      </c>
+      <c r="D72" s="327">
+        <v>1</v>
+      </c>
+      <c r="E72" s="326" t="s">
+        <v>148</v>
+      </c>
       <c r="F72" s="236"/>
       <c r="G72" s="237"/>
       <c r="H72" s="2"/>
@@ -14873,15 +14872,15 @@
       <c r="BL72" s="312"/>
       <c r="BM72" s="313"/>
       <c r="BN72" s="2"/>
-      <c r="BO72" s="329" t="s">
-        <v>205</v>
-      </c>
-      <c r="BP72" s="329"/>
-      <c r="BQ72" s="329"/>
-      <c r="BR72" s="329"/>
-      <c r="BS72" s="329"/>
-      <c r="BT72" s="329"/>
-      <c r="BU72" s="329"/>
+      <c r="BO72" s="332" t="s">
+        <v>199</v>
+      </c>
+      <c r="BP72" s="332"/>
+      <c r="BQ72" s="332"/>
+      <c r="BR72" s="332"/>
+      <c r="BS72" s="332"/>
+      <c r="BT72" s="332"/>
+      <c r="BU72" s="332"/>
       <c r="BV72" s="2"/>
       <c r="BW72" s="2"/>
       <c r="BX72" s="2"/>
@@ -14921,17 +14920,21 @@
       <c r="DF72" s="2"/>
     </row>
     <row r="73" spans="1:110" x14ac:dyDescent="0.8">
-      <c r="A73" s="2" t="s">
-        <v>194</v>
+      <c r="A73" s="281" t="s">
+        <v>189</v>
       </c>
       <c r="B73" s="291">
         <v>46129</v>
       </c>
       <c r="C73" s="235" t="s">
-        <v>85</v>
-      </c>
-      <c r="D73" s="235"/>
-      <c r="E73" s="235"/>
+        <v>84</v>
+      </c>
+      <c r="D73" s="327">
+        <v>1</v>
+      </c>
+      <c r="E73" s="326" t="s">
+        <v>148</v>
+      </c>
       <c r="F73" s="236"/>
       <c r="G73" s="237"/>
       <c r="H73" s="2"/>
@@ -14993,15 +14996,15 @@
       <c r="BL73" s="312"/>
       <c r="BM73" s="313"/>
       <c r="BN73" s="2"/>
-      <c r="BO73" s="329" t="s">
-        <v>206</v>
-      </c>
-      <c r="BP73" s="329"/>
-      <c r="BQ73" s="329"/>
-      <c r="BR73" s="329"/>
-      <c r="BS73" s="329"/>
-      <c r="BT73" s="329"/>
-      <c r="BU73" s="329"/>
+      <c r="BO73" s="332" t="s">
+        <v>200</v>
+      </c>
+      <c r="BP73" s="332"/>
+      <c r="BQ73" s="332"/>
+      <c r="BR73" s="332"/>
+      <c r="BS73" s="332"/>
+      <c r="BT73" s="332"/>
+      <c r="BU73" s="332"/>
       <c r="BV73" s="2"/>
       <c r="BW73" s="2"/>
       <c r="BX73" s="2"/>
@@ -15041,17 +15044,21 @@
       <c r="DF73" s="2"/>
     </row>
     <row r="74" spans="1:110" x14ac:dyDescent="0.8">
-      <c r="A74" s="2" t="s">
-        <v>193</v>
+      <c r="A74" s="281" t="s">
+        <v>188</v>
       </c>
       <c r="B74" s="291">
         <v>46129</v>
       </c>
       <c r="C74" s="235" t="s">
-        <v>85</v>
-      </c>
-      <c r="D74" s="235"/>
-      <c r="E74" s="235"/>
+        <v>84</v>
+      </c>
+      <c r="D74" s="327">
+        <v>1</v>
+      </c>
+      <c r="E74" s="326" t="s">
+        <v>148</v>
+      </c>
       <c r="F74" s="236"/>
       <c r="G74" s="237"/>
       <c r="H74" s="2"/>
@@ -15113,15 +15120,15 @@
       <c r="BL74" s="312"/>
       <c r="BM74" s="313"/>
       <c r="BN74" s="2"/>
-      <c r="BO74" s="329" t="s">
-        <v>207</v>
-      </c>
-      <c r="BP74" s="329"/>
-      <c r="BQ74" s="329"/>
-      <c r="BR74" s="329"/>
-      <c r="BS74" s="329"/>
-      <c r="BT74" s="329"/>
-      <c r="BU74" s="329"/>
+      <c r="BO74" s="332" t="s">
+        <v>201</v>
+      </c>
+      <c r="BP74" s="332"/>
+      <c r="BQ74" s="332"/>
+      <c r="BR74" s="332"/>
+      <c r="BS74" s="332"/>
+      <c r="BT74" s="332"/>
+      <c r="BU74" s="332"/>
       <c r="BV74" s="2"/>
       <c r="BW74" s="2"/>
       <c r="BX74" s="2"/>
@@ -15161,17 +15168,21 @@
       <c r="DF74" s="2"/>
     </row>
     <row r="75" spans="1:110" x14ac:dyDescent="0.8">
-      <c r="A75" s="2" t="s">
-        <v>192</v>
+      <c r="A75" s="281" t="s">
+        <v>187</v>
       </c>
       <c r="B75" s="291">
         <v>46129</v>
       </c>
       <c r="C75" s="235" t="s">
-        <v>85</v>
-      </c>
-      <c r="D75" s="238"/>
-      <c r="E75" s="238"/>
+        <v>84</v>
+      </c>
+      <c r="D75" s="329">
+        <v>1</v>
+      </c>
+      <c r="E75" s="326" t="s">
+        <v>148</v>
+      </c>
       <c r="F75" s="239"/>
       <c r="G75" s="240" t="s">
         <v>0</v>
@@ -15235,15 +15246,15 @@
       <c r="BL75" s="314"/>
       <c r="BM75" s="315"/>
       <c r="BN75" s="316"/>
-      <c r="BO75" s="329" t="s">
-        <v>208</v>
-      </c>
-      <c r="BP75" s="329"/>
-      <c r="BQ75" s="329"/>
-      <c r="BR75" s="329"/>
-      <c r="BS75" s="329"/>
-      <c r="BT75" s="329"/>
-      <c r="BU75" s="329"/>
+      <c r="BO75" s="332" t="s">
+        <v>202</v>
+      </c>
+      <c r="BP75" s="332"/>
+      <c r="BQ75" s="332"/>
+      <c r="BR75" s="332"/>
+      <c r="BS75" s="332"/>
+      <c r="BT75" s="332"/>
+      <c r="BU75" s="332"/>
       <c r="BV75" s="317"/>
       <c r="BW75" s="2"/>
       <c r="BX75" s="2"/>
@@ -15283,16 +15294,18 @@
       <c r="DF75" s="2"/>
     </row>
     <row r="76" spans="1:110" x14ac:dyDescent="0.8">
-      <c r="A76" s="2" t="s">
-        <v>210</v>
+      <c r="A76" s="432" t="s">
+        <v>209</v>
       </c>
       <c r="B76" s="291">
         <v>46129</v>
       </c>
       <c r="C76" s="235" t="s">
-        <v>85</v>
-      </c>
-      <c r="D76" s="238"/>
+        <v>84</v>
+      </c>
+      <c r="D76" s="329">
+        <v>0.75</v>
+      </c>
       <c r="E76" s="238"/>
       <c r="F76" s="239"/>
       <c r="G76" s="240"/>
@@ -15355,15 +15368,15 @@
       <c r="BL76" s="314"/>
       <c r="BM76" s="315"/>
       <c r="BN76" s="316"/>
-      <c r="BO76" s="329" t="s">
-        <v>211</v>
-      </c>
-      <c r="BP76" s="329"/>
-      <c r="BQ76" s="329"/>
-      <c r="BR76" s="329"/>
-      <c r="BS76" s="329"/>
-      <c r="BT76" s="329"/>
-      <c r="BU76" s="329"/>
+      <c r="BO76" s="433" t="s">
+        <v>204</v>
+      </c>
+      <c r="BP76" s="433"/>
+      <c r="BQ76" s="433"/>
+      <c r="BR76" s="433"/>
+      <c r="BS76" s="433"/>
+      <c r="BT76" s="433"/>
+      <c r="BU76" s="433"/>
       <c r="BV76" s="317"/>
       <c r="BW76" s="2"/>
       <c r="BX76" s="2"/>
@@ -15403,109 +15416,54 @@
       <c r="DF76" s="2"/>
     </row>
     <row r="77" spans="1:110" x14ac:dyDescent="0.8">
-      <c r="A77" s="2" t="s">
-        <v>174</v>
+      <c r="A77" s="281" t="s">
+        <v>186</v>
       </c>
       <c r="B77" s="291">
         <v>46129</v>
       </c>
       <c r="C77" s="235" t="s">
-        <v>85</v>
-      </c>
-      <c r="G77" s="240" t="s">
-        <v>0</v>
-      </c>
-      <c r="AT77" s="2"/>
-      <c r="AU77" s="2"/>
-      <c r="AV77" s="2"/>
-      <c r="AW77" s="2"/>
-      <c r="AX77" s="2"/>
-      <c r="AY77" s="2"/>
-      <c r="AZ77" s="2"/>
-      <c r="BA77" s="2"/>
-      <c r="BB77" s="2"/>
-      <c r="BC77" s="2"/>
-      <c r="BD77" s="2"/>
-      <c r="BE77" s="2"/>
-      <c r="BF77" s="2"/>
-      <c r="BG77" s="2"/>
-      <c r="BH77" s="2"/>
-      <c r="BI77" s="2"/>
-      <c r="BJ77" s="2"/>
-      <c r="BK77" s="2"/>
-      <c r="BL77" s="150"/>
-      <c r="BM77" s="318"/>
-      <c r="BN77" s="319"/>
-      <c r="BO77" s="329" t="s">
-        <v>181</v>
-      </c>
-      <c r="BP77" s="329"/>
-      <c r="BQ77" s="329"/>
-      <c r="BR77" s="329"/>
-      <c r="BS77" s="329"/>
-      <c r="BT77" s="329"/>
-      <c r="BU77" s="329"/>
-      <c r="BV77" s="320"/>
-      <c r="BW77" s="2"/>
-      <c r="BX77" s="2"/>
-      <c r="BY77" s="2"/>
-      <c r="BZ77" s="2"/>
-      <c r="CA77" s="2"/>
-      <c r="CB77" s="2"/>
-      <c r="CC77" s="2"/>
-      <c r="CD77" s="2"/>
-      <c r="CE77" s="2"/>
-      <c r="CF77" s="2"/>
-      <c r="CG77" s="2"/>
-      <c r="CH77" s="2"/>
-      <c r="CI77" s="2"/>
-      <c r="CJ77" s="2"/>
-      <c r="CK77" s="2"/>
-      <c r="CL77" s="2"/>
-      <c r="CM77" s="2"/>
-      <c r="CN77" s="2"/>
-      <c r="CO77" s="2"/>
-      <c r="CP77" s="2"/>
-      <c r="CQ77" s="2"/>
-      <c r="CR77" s="2"/>
-      <c r="CS77" s="2"/>
-      <c r="CT77" s="2"/>
-      <c r="CU77" s="2"/>
-      <c r="CV77" s="2"/>
-      <c r="CW77" s="2"/>
-      <c r="CX77" s="2"/>
-      <c r="CY77" s="2"/>
-      <c r="CZ77" s="2"/>
-      <c r="DA77" s="2"/>
-      <c r="DB77" s="2"/>
-      <c r="DC77" s="2"/>
-      <c r="DD77" s="2"/>
-      <c r="DE77" s="2"/>
-      <c r="DF77" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="D77" s="327">
+        <v>1</v>
+      </c>
+      <c r="E77" s="326" t="s">
+        <v>148</v>
+      </c>
+      <c r="BO77" s="332" t="s">
+        <v>205</v>
+      </c>
+      <c r="BP77" s="332"/>
+      <c r="BQ77" s="332"/>
+      <c r="BR77" s="332"/>
+      <c r="BS77" s="332"/>
+      <c r="BT77" s="332"/>
+      <c r="BU77" s="332"/>
     </row>
     <row r="78" spans="1:110" x14ac:dyDescent="0.8">
-      <c r="A78" s="2" t="s">
-        <v>191</v>
+      <c r="A78" s="435" t="s">
+        <v>210</v>
       </c>
       <c r="B78" s="291">
-        <v>46129</v>
-      </c>
-      <c r="C78" s="235" t="s">
-        <v>85</v>
-      </c>
-      <c r="BO78" s="329" t="s">
-        <v>212</v>
-      </c>
-      <c r="BP78" s="329"/>
-      <c r="BQ78" s="329"/>
-      <c r="BR78" s="329"/>
-      <c r="BS78" s="329"/>
-      <c r="BT78" s="329"/>
-      <c r="BU78" s="329"/>
+        <v>46134</v>
+      </c>
+      <c r="C78" s="291">
+        <v>46139</v>
+      </c>
+      <c r="BT78" s="436" t="s">
+        <v>211</v>
+      </c>
+      <c r="BU78" s="436"/>
+      <c r="BV78" s="436"/>
+      <c r="BW78" s="436"/>
+      <c r="BX78" s="436"/>
+      <c r="BY78" s="436"/>
     </row>
   </sheetData>
   <mergeCells count="78">
-    <mergeCell ref="BO78:BU78"/>
+    <mergeCell ref="BT78:BY78"/>
+    <mergeCell ref="BO77:BU77"/>
     <mergeCell ref="AF31:AM31"/>
     <mergeCell ref="CC2:DF2"/>
     <mergeCell ref="Y24:AF24"/>
@@ -15558,6 +15516,13 @@
     <mergeCell ref="BA50:BH50"/>
     <mergeCell ref="BA52:BH52"/>
     <mergeCell ref="BH69:BO69"/>
+    <mergeCell ref="BA53:BH53"/>
+    <mergeCell ref="BA55:BH55"/>
+    <mergeCell ref="BA54:BH54"/>
+    <mergeCell ref="BA56:BH56"/>
+    <mergeCell ref="BA51:BH51"/>
+    <mergeCell ref="BH57:BO57"/>
+    <mergeCell ref="BO76:BU76"/>
     <mergeCell ref="BO70:BS70"/>
     <mergeCell ref="BH62:BO62"/>
     <mergeCell ref="BH63:BO63"/>
@@ -15566,13 +15531,6 @@
     <mergeCell ref="BH66:BO66"/>
     <mergeCell ref="BH67:BO67"/>
     <mergeCell ref="BH68:BO68"/>
-    <mergeCell ref="BA53:BH53"/>
-    <mergeCell ref="BA55:BH55"/>
-    <mergeCell ref="BA54:BH54"/>
-    <mergeCell ref="BA56:BH56"/>
-    <mergeCell ref="BA51:BH51"/>
-    <mergeCell ref="BH57:BO57"/>
-    <mergeCell ref="BO77:BU77"/>
     <mergeCell ref="BH61:BO61"/>
     <mergeCell ref="BH60:BO60"/>
     <mergeCell ref="BH59:BO59"/>
@@ -15582,11 +15540,11 @@
     <mergeCell ref="BO72:BU72"/>
     <mergeCell ref="BO73:BU73"/>
     <mergeCell ref="BO74:BU74"/>
-    <mergeCell ref="BO76:BU76"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="G1:DF4 A1:C4 G5 I5:DF5 G6:I6 G8:DF10 X7:DF7 G7:J7 A8:C10 B7 B5:C5 A13:C13 A12 B15:C15 A11:B11 G23:DF23 S16:DF16 A14 A17:C17 A16:B16 G14:O14 S14:DF14 A23 G18:DF18 G21:Q21 S21:DF21 G15:Q17 S17:DF17 S6:DF6 A21:C21 C6 G33:AD33 B26:C26 G26:X26 AG26:DF26 A33 G32:AC32 AQ32:DF32 S15:DF15 AT77:BJ77 AF33:AN33 AU33:DF33 G34:AJ34 B34:C34 B39 G11:DF13 BT38:DF38 G38:AZ39 A70 BS39:DF39 AT69:AZ69 BQ69:DF69 AT70:BD70 BV70:DF70 G75:BK75 BW75:DF75 CA77:DF77 G69:AS70" numberStoredAsText="1"/>
+    <ignoredError sqref="G1:DF4 A1:C4 G5 I5:DF5 G6:I6 G8:DF10 X7:DF7 G7:J7 A8:C10 B7 B5:C5 A13:C13 A12 B15:C15 A11:B11 G23:DF23 S16:DF16 A14 A17:C17 A16:B16 G14:O14 S14:DF14 A23 G18:DF18 G21:Q21 S21:DF21 G15:Q17 S17:DF17 S6:DF6 A21:C21 C6 G33:AD33 B26:C26 G26:X26 AG26:DF26 A33 G32:AC32 AQ32:DF32 S15:DF15 AF33:AN33 AU33:DF33 G34:AJ34 B34:C34 B39 G11:DF13 BT38:DF38 G38:AZ39 BS39:DF39 AT69:AZ69 BQ69:DF69 AT70:BD70 BV70:DF70 G75:BK75 BW75:DF75 G69:AS70" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>